<commit_message>
Raise stability threshold from |r| >= 0.40 to |r| >= 0.50
A Pearson r of 0.50 means 25% of the variance in the MLB metric is
explained by the Asian-league metric — a meaningfully predictive
relationship. Updated threshold in build_analysis.py, generate_html.py,
and generate_excel.py.

With the stricter threshold:
- K/9 and BB/9 remain stable in 3/4 windows
- K/BB stable in 3/4 windows (career + 2yr + 3yr)
- WHIP stable in 2/4 windows (2yr + 3yr)
- ERA, HR/9 now stable in 0 windows
- GB% still stable in career (r=0.758, but only n=19)

Co-authored-by: colbymorris08 <colbymorris08@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/asian_pitcher_mlb_analysis.xlsx
+++ b/asian_pitcher_mlb_analysis.xlsx
@@ -5628,7 +5628,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Stable (|r|&gt;=0.40, p&lt;0.10)</t>
+          <t>Stable (|r|&gt;=0.50, p&lt;0.10)</t>
         </is>
       </c>
     </row>
@@ -5781,9 +5781,9 @@
       <c r="F6" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -5812,9 +5812,9 @@
       <c r="F7" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -5967,9 +5967,9 @@
       <c r="F12" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6029,9 +6029,9 @@
       <c r="F14" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6277,9 +6277,9 @@
       <c r="F22" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6587,9 +6587,9 @@
       <c r="F32" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6618,9 +6618,9 @@
       <c r="F33" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6804,9 +6804,9 @@
       <c r="F39" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -7114,9 +7114,9 @@
       <c r="F49" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -15742,7 +15742,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Threshold: |r| &gt;= 0.40 and p &lt; 0.10 to qualify as 'stable'</t>
+          <t>Threshold: |r| &gt;= 0.50 and p &lt; 0.10 to qualify as 'stable'</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add pitcher season table and correct four MLB IDs
The All pitchers view lists each transferred pitcher on two rows:
his last Asian season and his first MLB season. Stability and
Redundancy are styled as buttons.

Hideo Nomo, Hideki Irabu, Takashi Saito, and Chan Ho Park were
pointing at other players in the MLB Stats API. Their career and
season stats now use the correct IDs.

Co-authored-by: colbymorris08 <colbymorris08@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/asian_pitcher_mlb_analysis.xlsx
+++ b/asian_pitcher_mlb_analysis.xlsx
@@ -507,7 +507,7 @@
     <col width="7" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="8" customWidth="1" min="27" max="27"/>
-    <col width="7" customWidth="1" min="28" max="28"/>
+    <col width="8" customWidth="1" min="28" max="28"/>
     <col width="8" customWidth="1" min="29" max="29"/>
     <col width="8" customWidth="1" min="30" max="30"/>
     <col width="9" customWidth="1" min="31" max="31"/>
@@ -732,58 +732,58 @@
       </c>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n">
-        <v>2.66</v>
+        <v>4.24</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>884</v>
+        <v>1976.1</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>1.6</v>
+        <v>8.74</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1.17</v>
+        <v>4.14</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>0.09</v>
+        <v>1.14</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>1.173</v>
+        <v>1.354</v>
       </c>
       <c r="U2" s="2" t="n">
-        <v>1.37</v>
+        <v>2.11</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>0.414</v>
+        <v>0.53</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>38</v>
+        <v>43.9</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>10.3</v>
+        <v>21.8</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>41</v>
+        <v>123</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>58</v>
+        <v>109</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>103</v>
+        <v>323</v>
       </c>
       <c r="AD2" s="2" t="n">
-        <v>103</v>
+        <v>318</v>
       </c>
       <c r="AE2" s="2" t="n">
-        <v>157</v>
+        <v>1918</v>
       </c>
       <c r="AF2" s="2" t="n">
-        <v>115</v>
+        <v>908</v>
       </c>
       <c r="AG2" s="2" t="n">
         <v>0</v>
@@ -1053,61 +1053,61 @@
       </c>
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n">
-        <v>3.47</v>
+        <v>5.15</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>96</v>
+        <v>514</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>2.53</v>
+        <v>7.09</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>3.28</v>
+        <v>3.06</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>0.19</v>
+        <v>1.59</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>1.344</v>
+        <v>1.405</v>
       </c>
       <c r="U5" s="2" t="n">
-        <v>0.77</v>
+        <v>2.31</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>0.3</v>
+        <v>0.493</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>36</v>
+        <v>45.4</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>0.2</v>
+        <v>3.4</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="AC5" s="2" t="n">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="AD5" s="2" t="n">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="AE5" s="2" t="n">
-        <v>27</v>
+        <v>405</v>
       </c>
       <c r="AF5" s="2" t="n">
-        <v>35</v>
+        <v>175</v>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -1592,61 +1592,61 @@
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n">
-        <v>4.07</v>
+        <v>2.34</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>1189.1</v>
+        <v>338</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>6.92</v>
+        <v>10.65</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>2.78</v>
+        <v>2.88</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>0.99</v>
+        <v>0.67</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>1.384</v>
+        <v>1.059</v>
       </c>
       <c r="U10" s="2" t="n">
-        <v>2.49</v>
+        <v>3.7</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>0.504</v>
+        <v>0.583</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>59</v>
+        <v>44.2</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>86</v>
+        <v>185</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>6.9</v>
+        <v>10.5</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>68</v>
+        <v>15</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>211</v>
+        <v>338</v>
       </c>
       <c r="AD10" s="2" t="n">
-        <v>197</v>
+        <v>0</v>
       </c>
       <c r="AE10" s="2" t="n">
-        <v>914</v>
+        <v>400</v>
       </c>
       <c r="AF10" s="2" t="n">
-        <v>367</v>
+        <v>108</v>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
@@ -3595,61 +3595,61 @@
       </c>
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n">
-        <v>4.5</v>
+        <v>4.36</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>2</v>
+        <v>1993</v>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>7.4</v>
+        <v>7.74</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>4.5</v>
+        <v>4.11</v>
       </c>
       <c r="S29" s="2" t="n">
-        <v>1.2</v>
+        <v>1.04</v>
       </c>
       <c r="T29" s="2" t="n">
-        <v>1.5</v>
+        <v>1.396</v>
       </c>
       <c r="U29" s="2" t="n">
-        <v>2.06</v>
+        <v>1.88</v>
       </c>
       <c r="V29" s="2" t="n">
         <v>0.5590000000000001</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>38</v>
+        <v>51.7</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>0</v>
+        <v>18.1</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="AA29" s="2" t="n">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="AB29" s="2" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="AC29" s="2" t="n">
-        <v>1</v>
+        <v>476</v>
       </c>
       <c r="AD29" s="2" t="n">
-        <v>0</v>
+        <v>287</v>
       </c>
       <c r="AE29" s="2" t="n">
-        <v>0</v>
+        <v>1715</v>
       </c>
       <c r="AF29" s="2" t="n">
-        <v>1</v>
+        <v>910</v>
       </c>
       <c r="AG29" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -5649,13 +5649,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.395</v>
+        <v>0.19</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.023</v>
+        <v>0.2749</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -5680,13 +5680,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.623</v>
+        <v>0.545</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.0001</v>
+        <v>0.0007</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
@@ -5711,13 +5711,13 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.593</v>
+        <v>0.513</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0003</v>
+        <v>0.0016</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
@@ -5742,13 +5742,13 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.343</v>
+        <v>0.112</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0506</v>
+        <v>0.52</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -5773,13 +5773,13 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.418</v>
+        <v>0.127</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0155</v>
+        <v>0.4678</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -5804,13 +5804,13 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.439</v>
+        <v>0.381</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0106</v>
+        <v>0.0239</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -5835,13 +5835,13 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.353</v>
+        <v>0.048</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.0409</v>
+        <v>0.782</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -5866,17 +5866,17 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.513</v>
+        <v>0.412</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0125</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>36</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -5897,13 +5897,13 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.674</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
@@ -5928,13 +5928,13 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>-0.032</v>
+        <v>-0.125</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.8584000000000001</v>
+        <v>0.4664</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -5959,13 +5959,13 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.483</v>
+        <v>0.103</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0038</v>
+        <v>0.5487</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -5990,13 +5990,13 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.611</v>
+        <v>0.508</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0001</v>
+        <v>0.0015</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -6021,13 +6021,13 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.461</v>
+        <v>0.277</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0047</v>
+        <v>0.0922</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -6052,17 +6052,17 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.442</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.0004</v>
+        <v>0.0055</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>38</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6083,13 +6083,13 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.727</v>
+        <v>0.651</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -6114,13 +6114,13 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.18</v>
+        <v>0.005</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.2939</v>
+        <v>0.9782999999999999</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -6145,17 +6145,17 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.593</v>
+        <v>0.399</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0001</v>
+        <v>0.013</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>38</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6176,13 +6176,13 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.634</v>
+        <v>0.58</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
@@ -6207,10 +6207,10 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.168</v>
+        <v>0.141</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.2697</v>
+        <v>0.3559</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>45</v>
@@ -6238,17 +6238,17 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.349</v>
+        <v>0.526</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.0187</v>
+        <v>0.0002</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -6269,17 +6269,17 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.439</v>
+        <v>0.616</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.0026</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -6300,10 +6300,10 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>-0.151</v>
+        <v>-0.272</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.321</v>
+        <v>0.0703</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>45</v>
@@ -6331,10 +6331,10 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.386</v>
+        <v>0.369</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0089</v>
+        <v>0.0126</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>45</v>
@@ -6362,17 +6362,17 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.519</v>
+        <v>0.493</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6424,13 +6424,13 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.396</v>
+        <v>0.116</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0498</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -6455,13 +6455,13 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.773</v>
+        <v>0.676</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
@@ -6486,13 +6486,13 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.614</v>
+        <v>0.517</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0057</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
@@ -6517,13 +6517,13 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.377</v>
+        <v>0.068</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0636</v>
+        <v>0.736</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -6548,17 +6548,17 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.525</v>
+        <v>0.117</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.007</v>
+        <v>0.5615</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>27</v>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6579,13 +6579,13 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.431</v>
+        <v>0.379</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0314</v>
+        <v>0.0512</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -6610,13 +6610,13 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.4</v>
+        <v>0.002</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0429</v>
+        <v>0.9938</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -6641,17 +6641,17 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.618</v>
+        <v>0.493</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.0008</v>
+        <v>0.0077</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>28</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6672,13 +6672,13 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.77</v>
+        <v>0.652</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
@@ -6703,13 +6703,13 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.041</v>
+        <v>-0.111</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.8431</v>
+        <v>0.5752</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -6734,17 +6734,17 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.517</v>
+        <v>0.055</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0069</v>
+        <v>0.7805</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>28</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6765,13 +6765,13 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.678</v>
+        <v>0.572</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.0001</v>
+        <v>0.0015</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -6796,13 +6796,13 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.448</v>
+        <v>0.199</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.0191</v>
+        <v>0.3017</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -6827,13 +6827,13 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.679</v>
+        <v>0.524</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.0001</v>
+        <v>0.0035</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
@@ -6858,13 +6858,13 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.832</v>
+        <v>0.75</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
@@ -6889,13 +6889,13 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.324</v>
+        <v>0.017</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.0988</v>
+        <v>0.929</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -6920,17 +6920,17 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.618</v>
+        <v>0.375</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0448</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>29</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6951,13 +6951,13 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.711</v>
+        <v>0.656</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -6982,10 +6982,10 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.065</v>
+        <v>0.045</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.7272999999999999</v>
+        <v>0.8083</v>
       </c>
       <c r="F45" s="2" t="n">
         <v>31</v>
@@ -7013,17 +7013,17 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0.303</v>
+        <v>0.547</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0014</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -7044,10 +7044,10 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0.518</v>
+        <v>0.737</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.0029</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>31</v>
@@ -7075,10 +7075,10 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>-0.041</v>
+        <v>-0.203</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.8284</v>
+        <v>0.2726</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>31</v>
@@ -7106,10 +7106,10 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.449</v>
+        <v>0.455</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.0113</v>
+        <v>0.0101</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>31</v>
@@ -7137,10 +7137,10 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.609</v>
+        <v>0.575</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.0003</v>
+        <v>0.0007</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>31</v>
@@ -7757,10 +7757,10 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.19</v>
+        <v>0.175</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.5331</v>
+        <v>0.5685</v>
       </c>
       <c r="F70" s="2" t="n">
         <v>13</v>
@@ -7788,10 +7788,10 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.534</v>
+        <v>0.506</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>0.0604</v>
+        <v>0.07770000000000001</v>
       </c>
       <c r="F71" s="2" t="n">
         <v>13</v>
@@ -7819,10 +7819,10 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.312</v>
+        <v>0.291</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.2996</v>
+        <v>0.3339</v>
       </c>
       <c r="F72" s="2" t="n">
         <v>13</v>
@@ -7850,10 +7850,10 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>-0.296</v>
+        <v>-0.331</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>0.326</v>
+        <v>0.2701</v>
       </c>
       <c r="F73" s="2" t="n">
         <v>13</v>
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0.201</v>
+        <v>0.145</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.5108</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="F74" s="2" t="n">
         <v>13</v>
@@ -7912,10 +7912,10 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>0.322</v>
+        <v>0.338</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>0.2839</v>
+        <v>0.2592</v>
       </c>
       <c r="F75" s="2" t="n">
         <v>13</v>
@@ -8041,14 +8041,14 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.066</v>
+        <v>0.175</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.7019</v>
+        <v>0.3079</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>36</v>
@@ -8077,14 +8077,14 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.055</v>
+        <v>0.112</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.7518</v>
+        <v>0.5152</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>36</v>
@@ -8113,14 +8113,14 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.041</v>
+        <v>-0.094</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.8127</v>
+        <v>0.5854</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>36</v>
@@ -8149,14 +8149,14 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.032</v>
+        <v>0.058</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.8548</v>
+        <v>0.7359</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>36</v>
@@ -8185,14 +8185,14 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-0.031</v>
+        <v>-0.024</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.8575</v>
+        <v>0.8882</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>36</v>
@@ -8221,14 +8221,14 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-0.023</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.8923</v>
+        <v>0.9573</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>36</v>
@@ -8261,10 +8261,10 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.222</v>
+        <v>0.134</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.1932</v>
+        <v>0.4372</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>36</v>
@@ -8293,14 +8293,14 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.214</v>
+        <v>-0.073</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.2102</v>
+        <v>0.6728</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>36</v>
@@ -8329,14 +8329,14 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-0.135</v>
+        <v>-0.04</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.434</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>36</v>
@@ -8365,14 +8365,14 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-0.102</v>
+        <v>0.023</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.5548999999999999</v>
+        <v>0.8925</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>36</v>
@@ -8401,14 +8401,14 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-0.042</v>
+        <v>-0.016</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.8095</v>
+        <v>0.9272</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>36</v>
@@ -8437,14 +8437,14 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-0</v>
+        <v>0.01</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.9993</v>
+        <v>0.9534</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>36</v>
@@ -8689,14 +8689,14 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>-0.241</v>
+        <v>0.224</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.1512</v>
+        <v>0.1827</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>37</v>
@@ -8725,14 +8725,14 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.179</v>
+        <v>-0.2</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.2878</v>
+        <v>0.2352</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>37</v>
@@ -8761,14 +8761,14 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>-0.157</v>
+        <v>0.134</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.3522</v>
+        <v>0.4303</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>37</v>
@@ -8797,14 +8797,14 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>-0.153</v>
+        <v>-0.091</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.3669</v>
+        <v>0.5911</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>37</v>
@@ -8833,14 +8833,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>-0.037</v>
+        <v>-0.014</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.8263</v>
+        <v>0.9334</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>37</v>
@@ -8869,14 +8869,14 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>-0.014</v>
+        <v>-0.011</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.9351</v>
+        <v>0.9477</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>37</v>
@@ -8905,21 +8905,21 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>-0.318</v>
+        <v>-0.185</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.0547</v>
+        <v>0.2727</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -8945,17 +8945,17 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.282</v>
+        <v>0.183</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.279</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -8977,14 +8977,14 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>-0.214</v>
+        <v>-0.156</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.2042</v>
+        <v>0.3554</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>37</v>
@@ -9013,14 +9013,14 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>-0.174</v>
+        <v>-0.094</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.3025</v>
+        <v>0.5814</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>37</v>
@@ -9049,14 +9049,14 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>-0.173</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.3057</v>
+        <v>0.6084000000000001</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>37</v>
@@ -9085,14 +9085,14 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>-0.139</v>
+        <v>-0.053</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.412</v>
+        <v>0.7547</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>37</v>
@@ -9337,21 +9337,21 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>-0.242</v>
+        <v>0.281</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.1378</v>
+        <v>0.0827</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -9373,14 +9373,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.225</v>
+        <v>-0.206</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.1689</v>
+        <v>0.2083</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>39</v>
@@ -9409,14 +9409,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>-0.196</v>
+        <v>0.187</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.2328</v>
+        <v>0.255</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>39</v>
@@ -9445,14 +9445,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>-0.138</v>
+        <v>-0.09</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.401</v>
+        <v>0.5867</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>39</v>
@@ -9481,14 +9481,14 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>-0.044</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.6087</v>
+        <v>0.7903</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>39</v>
@@ -9517,14 +9517,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.01</v>
+        <v>-0.024</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.9529</v>
+        <v>0.8865</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>39</v>
@@ -9553,21 +9553,21 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>-0.315</v>
+        <v>-0.211</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.0509</v>
+        <v>0.1972</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -9589,14 +9589,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.247</v>
+        <v>-0.171</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.1289</v>
+        <v>0.2977</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>39</v>
@@ -9625,14 +9625,14 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>-0.236</v>
+        <v>0.158</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0.1481</v>
+        <v>0.3358</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>39</v>
@@ -9661,14 +9661,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>-0.222</v>
+        <v>-0.15</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.1736</v>
+        <v>0.3617</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>39</v>
@@ -9697,14 +9697,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>-0.213</v>
+        <v>-0.132</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.1935</v>
+        <v>0.4237</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>39</v>
@@ -9733,14 +9733,14 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>-0.175</v>
+        <v>-0.125</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.286</v>
+        <v>0.4494</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>39</v>
@@ -9989,10 +9989,10 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.103</v>
+        <v>0.225</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.5012</v>
+        <v>0.1365</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>45</v>
@@ -10025,10 +10025,10 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>-0.074</v>
+        <v>-0.145</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.6297</v>
+        <v>0.3427</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>45</v>
@@ -10061,10 +10061,10 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.081</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.6449</v>
+        <v>0.5959</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>45</v>
@@ -10097,10 +10097,10 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>-0.051</v>
+        <v>-0.062</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.739</v>
+        <v>0.6843</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>45</v>
@@ -10129,14 +10129,14 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>-0.05</v>
+        <v>-0.048</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.745</v>
+        <v>0.7524</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>45</v>
@@ -10165,17 +10165,17 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>GB%</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>-0.022</v>
+        <v>-0.018</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.8856000000000001</v>
+        <v>0.9409</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -10201,17 +10201,17 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>GB%</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>-0.018</v>
+        <v>-0.014</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.9409</v>
+        <v>0.9248</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -10237,21 +10237,21 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>GB%</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>-0.255</v>
+        <v>0.226</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.0912</v>
+        <v>0.3529</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>19</v>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -10273,17 +10273,17 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>GB%</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.226</v>
+        <v>-0.179</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.3529</v>
+        <v>0.239</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -10309,14 +10309,14 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>-0.182</v>
+        <v>-0.103</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.2325</v>
+        <v>0.4994</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>45</v>
@@ -10345,14 +10345,14 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>-0.163</v>
+        <v>-0.04</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.2852</v>
+        <v>0.7946</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>45</v>
@@ -10381,14 +10381,14 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.151</v>
+        <v>-0.039</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.3205</v>
+        <v>0.7982</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>45</v>
@@ -10417,14 +10417,14 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>-0.125</v>
+        <v>-0.033</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.4119</v>
+        <v>0.8310999999999999</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>45</v>
@@ -10453,14 +10453,14 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>-0.125</v>
+        <v>0.027</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.4151</v>
+        <v>0.861</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>45</v>
@@ -10741,14 +10741,14 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.092</v>
+        <v>0.182</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.6411</v>
+        <v>0.3548</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>28</v>
@@ -10781,10 +10781,10 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.037</v>
+        <v>0.156</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.8504</v>
+        <v>0.4267</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>28</v>
@@ -10813,14 +10813,14 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>0.034</v>
+        <v>0.098</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>0.8629</v>
+        <v>0.6204</v>
       </c>
       <c r="G79" s="2" t="n">
         <v>28</v>
@@ -10849,14 +10849,14 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.034</v>
+        <v>-0.079</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0.8619</v>
+        <v>0.6893</v>
       </c>
       <c r="G80" s="2" t="n">
         <v>28</v>
@@ -10885,14 +10885,14 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>0.026</v>
+        <v>0.011</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>0.8949</v>
+        <v>0.9542</v>
       </c>
       <c r="G81" s="2" t="n">
         <v>28</v>
@@ -10921,14 +10921,14 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>0.013</v>
+        <v>0.007</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>0.9494</v>
+        <v>0.9716</v>
       </c>
       <c r="G82" s="2" t="n">
         <v>28</v>
@@ -10957,14 +10957,14 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>-0.279</v>
+        <v>0.169</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.1498</v>
+        <v>0.3912</v>
       </c>
       <c r="G83" s="2" t="n">
         <v>28</v>
@@ -10993,14 +10993,14 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>0.274</v>
+        <v>-0.146</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>0.1588</v>
+        <v>0.4573</v>
       </c>
       <c r="G84" s="2" t="n">
         <v>28</v>
@@ -11029,14 +11029,14 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>-0.188</v>
+        <v>-0.079</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>0.3373</v>
+        <v>0.6904</v>
       </c>
       <c r="G85" s="2" t="n">
         <v>28</v>
@@ -11069,10 +11069,10 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>-0.08500000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0.6677</v>
+        <v>0.7251</v>
       </c>
       <c r="G86" s="2" t="n">
         <v>28</v>
@@ -11101,14 +11101,14 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>-0.059</v>
+        <v>0.063</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>0.7648</v>
+        <v>0.7503</v>
       </c>
       <c r="G87" s="2" t="n">
         <v>28</v>
@@ -11137,14 +11137,14 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>-0.011</v>
+        <v>-0.029</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>0.9552</v>
+        <v>0.8853</v>
       </c>
       <c r="G88" s="2" t="n">
         <v>28</v>
@@ -11389,14 +11389,14 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>-0.299</v>
+        <v>-0.228</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.1149</v>
+        <v>0.2347</v>
       </c>
       <c r="G95" s="2" t="n">
         <v>29</v>
@@ -11425,14 +11425,14 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>-0.277</v>
+        <v>0.168</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.1455</v>
+        <v>0.3831</v>
       </c>
       <c r="G96" s="2" t="n">
         <v>29</v>
@@ -11461,14 +11461,14 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>0.23</v>
+        <v>0.158</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>0.2293</v>
+        <v>0.4128</v>
       </c>
       <c r="G97" s="2" t="n">
         <v>29</v>
@@ -11497,14 +11497,14 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>-0.174</v>
+        <v>-0.077</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>0.3677</v>
+        <v>0.6921</v>
       </c>
       <c r="G98" s="2" t="n">
         <v>29</v>
@@ -11533,14 +11533,14 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>-0.172</v>
+        <v>-0.077</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>0.3718</v>
+        <v>0.6927</v>
       </c>
       <c r="G99" s="2" t="n">
         <v>29</v>
@@ -11569,14 +11569,14 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>0.017</v>
+        <v>-0.006</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>0.9286</v>
+        <v>0.9748</v>
       </c>
       <c r="G100" s="2" t="n">
         <v>29</v>
@@ -11605,21 +11605,21 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>-0.403</v>
+        <v>-0.261</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>0.0303</v>
+        <v>0.171</v>
       </c>
       <c r="G101" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H101" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -11645,17 +11645,17 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>0.337</v>
+        <v>0.221</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>0.0741</v>
+        <v>0.2504</v>
       </c>
       <c r="G102" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H102" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -11677,14 +11677,14 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>-0.298</v>
+        <v>-0.219</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>0.1162</v>
+        <v>0.2527</v>
       </c>
       <c r="G103" s="2" t="n">
         <v>29</v>
@@ -11713,14 +11713,14 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>-0.208</v>
+        <v>-0.136</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>0.2792</v>
+        <v>0.4824</v>
       </c>
       <c r="G104" s="2" t="n">
         <v>29</v>
@@ -11749,14 +11749,14 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.106</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>0.2985</v>
+        <v>0.585</v>
       </c>
       <c r="G105" s="2" t="n">
         <v>29</v>
@@ -11789,10 +11789,10 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>-0.184</v>
+        <v>-0.034</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>0.3401</v>
+        <v>0.8627</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>29</v>
@@ -12037,14 +12037,14 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>-0.267</v>
+        <v>0.253</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>0.1543</v>
+        <v>0.1767</v>
       </c>
       <c r="G113" s="2" t="n">
         <v>30</v>
@@ -12073,14 +12073,14 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>0.263</v>
+        <v>-0.221</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>0.1602</v>
+        <v>0.2412</v>
       </c>
       <c r="G114" s="2" t="n">
         <v>30</v>
@@ -12109,14 +12109,14 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>-0.246</v>
+        <v>0.212</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0.1894</v>
+        <v>0.2603</v>
       </c>
       <c r="G115" s="2" t="n">
         <v>30</v>
@@ -12145,14 +12145,14 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>-0.135</v>
+        <v>-0.116</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>0.4777</v>
+        <v>0.5399</v>
       </c>
       <c r="G116" s="2" t="n">
         <v>30</v>
@@ -12181,14 +12181,14 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>0.134</v>
+        <v>0.013</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0.481</v>
+        <v>0.9456</v>
       </c>
       <c r="G117" s="2" t="n">
         <v>30</v>
@@ -12217,14 +12217,14 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>-0.091</v>
+        <v>-0.002</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>0.6321</v>
+        <v>0.9897</v>
       </c>
       <c r="G118" s="2" t="n">
         <v>30</v>
@@ -12253,21 +12253,21 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>-0.41</v>
+        <v>-0.258</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>0.0245</v>
+        <v>0.1692</v>
       </c>
       <c r="G119" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H119" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -12289,21 +12289,21 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>0.324</v>
+        <v>-0.248</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>0.0804</v>
+        <v>0.1861</v>
       </c>
       <c r="G120" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H120" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -12325,14 +12325,14 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>-0.29</v>
+        <v>0.221</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>0.1205</v>
+        <v>0.241</v>
       </c>
       <c r="G121" s="2" t="n">
         <v>30</v>
@@ -12361,14 +12361,14 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>-0.26</v>
+        <v>-0.154</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>0.1652</v>
+        <v>0.4167</v>
       </c>
       <c r="G122" s="2" t="n">
         <v>30</v>
@@ -12397,14 +12397,14 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>-0.234</v>
+        <v>-0.135</v>
       </c>
       <c r="F123" s="2" t="n">
-        <v>0.2124</v>
+        <v>0.4757</v>
       </c>
       <c r="G123" s="2" t="n">
         <v>30</v>
@@ -12437,10 +12437,10 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>-0.182</v>
+        <v>-0.13</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>0.3347</v>
+        <v>0.4933</v>
       </c>
       <c r="G124" s="2" t="n">
         <v>30</v>
@@ -12685,17 +12685,17 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>GB%</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>-0.223</v>
+        <v>-0.249</v>
       </c>
       <c r="F131" s="2" t="n">
-        <v>0.4444</v>
+        <v>0.177</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -12721,17 +12721,17 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>GB%</t>
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>0.217</v>
+        <v>-0.223</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>0.2404</v>
+        <v>0.4444</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -12757,14 +12757,14 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>-0.176</v>
+        <v>0.219</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>0.3431</v>
+        <v>0.236</v>
       </c>
       <c r="G133" s="2" t="n">
         <v>31</v>
@@ -12793,14 +12793,14 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>-0.172</v>
+        <v>0.191</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>0.3547</v>
+        <v>0.3042</v>
       </c>
       <c r="G134" s="2" t="n">
         <v>31</v>
@@ -12829,14 +12829,14 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E135" s="2" t="n">
-        <v>-0.055</v>
+        <v>-0.13</v>
       </c>
       <c r="F135" s="2" t="n">
-        <v>0.7694</v>
+        <v>0.4872</v>
       </c>
       <c r="G135" s="2" t="n">
         <v>31</v>
@@ -12865,14 +12865,14 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>0.035</v>
+        <v>0.074</v>
       </c>
       <c r="F136" s="2" t="n">
-        <v>0.8517</v>
+        <v>0.6922</v>
       </c>
       <c r="G136" s="2" t="n">
         <v>31</v>
@@ -12901,14 +12901,14 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>0.008</v>
+        <v>-0.051</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>0.966</v>
+        <v>0.7871</v>
       </c>
       <c r="G137" s="2" t="n">
         <v>31</v>
@@ -12941,17 +12941,17 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>-0.342</v>
+        <v>-0.196</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>0.0595</v>
+        <v>0.2895</v>
       </c>
       <c r="G138" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="H138" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -12973,14 +12973,14 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E139" s="2" t="n">
-        <v>-0.268</v>
+        <v>-0.181</v>
       </c>
       <c r="F139" s="2" t="n">
-        <v>0.1445</v>
+        <v>0.3311</v>
       </c>
       <c r="G139" s="2" t="n">
         <v>31</v>
@@ -13009,14 +13009,14 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>-0.236</v>
+        <v>-0.176</v>
       </c>
       <c r="F140" s="2" t="n">
-        <v>0.2012</v>
+        <v>0.3446</v>
       </c>
       <c r="G140" s="2" t="n">
         <v>31</v>
@@ -13049,10 +13049,10 @@
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>-0.23</v>
+        <v>-0.175</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>0.2134</v>
+        <v>0.3456</v>
       </c>
       <c r="G141" s="2" t="n">
         <v>31</v>
@@ -13081,14 +13081,14 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>0.208</v>
+        <v>-0.147</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0.2618</v>
+        <v>0.4288</v>
       </c>
       <c r="G142" s="2" t="n">
         <v>31</v>
@@ -13117,14 +13117,14 @@
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E143" s="2" t="n">
-        <v>-0.179</v>
+        <v>0.13</v>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0.3348</v>
+        <v>0.4852</v>
       </c>
       <c r="G143" s="2" t="n">
         <v>31</v>
@@ -14777,10 +14777,10 @@
         </is>
       </c>
       <c r="E189" s="2" t="n">
-        <v>0.269</v>
+        <v>0.217</v>
       </c>
       <c r="F189" s="2" t="n">
-        <v>0.375</v>
+        <v>0.4762</v>
       </c>
       <c r="G189" s="2" t="n">
         <v>13</v>
@@ -14813,10 +14813,10 @@
         </is>
       </c>
       <c r="E190" s="2" t="n">
-        <v>0.248</v>
+        <v>0.209</v>
       </c>
       <c r="F190" s="2" t="n">
-        <v>0.4136</v>
+        <v>0.4939</v>
       </c>
       <c r="G190" s="2" t="n">
         <v>13</v>
@@ -14849,10 +14849,10 @@
         </is>
       </c>
       <c r="E191" s="2" t="n">
-        <v>-0.225</v>
+        <v>-0.176</v>
       </c>
       <c r="F191" s="2" t="n">
-        <v>0.4594</v>
+        <v>0.5662</v>
       </c>
       <c r="G191" s="2" t="n">
         <v>13</v>
@@ -14881,14 +14881,14 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E192" s="2" t="n">
-        <v>-0.129</v>
+        <v>-0.082</v>
       </c>
       <c r="F192" s="2" t="n">
-        <v>0.6746</v>
+        <v>0.7902</v>
       </c>
       <c r="G192" s="2" t="n">
         <v>13</v>
@@ -14917,14 +14917,14 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E193" s="2" t="n">
-        <v>0.103</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="F193" s="2" t="n">
-        <v>0.7373</v>
+        <v>0.8151</v>
       </c>
       <c r="G193" s="2" t="n">
         <v>13</v>
@@ -14953,14 +14953,14 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E194" s="2" t="n">
-        <v>-0.033</v>
+        <v>0.056</v>
       </c>
       <c r="F194" s="2" t="n">
-        <v>0.9137999999999999</v>
+        <v>0.8569</v>
       </c>
       <c r="G194" s="2" t="n">
         <v>13</v>
@@ -15025,14 +15025,14 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E196" s="2" t="n">
-        <v>0.06</v>
+        <v>0.274</v>
       </c>
       <c r="F196" s="2" t="n">
-        <v>0.8447</v>
+        <v>0.3645</v>
       </c>
       <c r="G196" s="2" t="n">
         <v>13</v>
@@ -15065,10 +15065,10 @@
         </is>
       </c>
       <c r="E197" s="2" t="n">
-        <v>0.039</v>
+        <v>0.264</v>
       </c>
       <c r="F197" s="2" t="n">
-        <v>0.8993</v>
+        <v>0.3836</v>
       </c>
       <c r="G197" s="2" t="n">
         <v>13</v>
@@ -15097,14 +15097,14 @@
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E198" s="2" t="n">
-        <v>0.035</v>
+        <v>0.256</v>
       </c>
       <c r="F198" s="2" t="n">
-        <v>0.9092</v>
+        <v>0.3982</v>
       </c>
       <c r="G198" s="2" t="n">
         <v>13</v>
@@ -15133,14 +15133,14 @@
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E199" s="2" t="n">
-        <v>0.021</v>
+        <v>-0.223</v>
       </c>
       <c r="F199" s="2" t="n">
-        <v>0.9445</v>
+        <v>0.4634</v>
       </c>
       <c r="G199" s="2" t="n">
         <v>13</v>
@@ -15169,14 +15169,14 @@
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E200" s="2" t="n">
-        <v>0.019</v>
+        <v>-0.218</v>
       </c>
       <c r="F200" s="2" t="n">
-        <v>0.9518</v>
+        <v>0.475</v>
       </c>
       <c r="G200" s="2" t="n">
         <v>13</v>
@@ -15205,14 +15205,14 @@
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E201" s="2" t="n">
-        <v>0.008</v>
+        <v>0.196</v>
       </c>
       <c r="F201" s="2" t="n">
-        <v>0.9797</v>
+        <v>0.5217000000000001</v>
       </c>
       <c r="G201" s="2" t="n">
         <v>13</v>

</xml_diff>

<commit_message>
Add Asian seasons for the American returnees left out of the sample.
Nick Martinez, Kyle Hart, Drew Anderson, Aaron Brooks, Ryan Weiss, and Chris Martin had MLB rows but no register page, so they were marked omitted. Their NPB and KBO seasons are now in the correlations.

Co-authored-by: colbymorris08 <colbymorris08@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/asian_pitcher_mlb_analysis.xlsx
+++ b/asian_pitcher_mlb_analysis.xlsx
@@ -7918,14 +7918,30 @@
       <c r="E70" s="2" t="n">
         <v>2018</v>
       </c>
-      <c r="F70" s="2" t="n"/>
-      <c r="G70" s="2" t="n"/>
-      <c r="H70" s="2" t="n"/>
-      <c r="I70" s="2" t="n"/>
-      <c r="J70" s="2" t="n"/>
-      <c r="K70" s="2" t="n"/>
-      <c r="L70" s="2" t="n"/>
-      <c r="M70" s="2" t="n"/>
+      <c r="F70" s="2" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>0.675</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>0.5</v>
+      </c>
       <c r="N70" s="2" t="n"/>
       <c r="O70" s="2" t="n">
         <v>3.53</v>
@@ -8116,14 +8132,30 @@
       <c r="E72" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F72" s="2" t="n"/>
-      <c r="G72" s="2" t="n"/>
-      <c r="H72" s="2" t="n"/>
-      <c r="I72" s="2" t="n"/>
-      <c r="J72" s="2" t="n"/>
-      <c r="K72" s="2" t="n"/>
-      <c r="L72" s="2" t="n"/>
-      <c r="M72" s="2" t="n"/>
+      <c r="F72" s="2" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>377.4</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>1.245</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>0.5</v>
+      </c>
       <c r="N72" s="2" t="n"/>
       <c r="O72" s="2" t="n">
         <v>3.99</v>
@@ -8528,14 +8560,30 @@
       <c r="E76" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="F76" s="2" t="n"/>
-      <c r="G76" s="2" t="n"/>
-      <c r="H76" s="2" t="n"/>
-      <c r="I76" s="2" t="n"/>
-      <c r="J76" s="2" t="n"/>
-      <c r="K76" s="2" t="n"/>
-      <c r="L76" s="2" t="n"/>
-      <c r="M76" s="2" t="n"/>
+      <c r="F76" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>1.032</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>0.8129999999999999</v>
+      </c>
       <c r="N76" s="2" t="n"/>
       <c r="O76" s="2" t="n">
         <v>6.25</v>
@@ -8833,14 +8881,30 @@
       <c r="E79" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F79" s="2" t="n"/>
-      <c r="G79" s="2" t="n"/>
-      <c r="H79" s="2" t="n"/>
-      <c r="I79" s="2" t="n"/>
-      <c r="J79" s="2" t="n"/>
-      <c r="K79" s="2" t="n"/>
-      <c r="L79" s="2" t="n"/>
-      <c r="M79" s="2" t="n"/>
+      <c r="F79" s="2" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>229.1</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>1.152</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>0.529</v>
+      </c>
       <c r="N79" s="2" t="n"/>
       <c r="O79" s="2" t="n">
         <v>6.48</v>
@@ -9031,14 +9095,30 @@
       <c r="E81" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="F81" s="2" t="n"/>
-      <c r="G81" s="2" t="n"/>
-      <c r="H81" s="2" t="n"/>
-      <c r="I81" s="2" t="n"/>
-      <c r="J81" s="2" t="n"/>
-      <c r="K81" s="2" t="n"/>
-      <c r="L81" s="2" t="n"/>
-      <c r="M81" s="2" t="n"/>
+      <c r="F81" s="2" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>401.4</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>1.131</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>0.667</v>
+      </c>
       <c r="N81" s="2" t="n"/>
       <c r="O81" s="2" t="n">
         <v>4.49</v>
@@ -9122,14 +9202,30 @@
       <c r="E82" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="F82" s="2" t="n"/>
-      <c r="G82" s="2" t="n"/>
-      <c r="H82" s="2" t="n"/>
-      <c r="I82" s="2" t="n"/>
-      <c r="J82" s="2" t="n"/>
-      <c r="K82" s="2" t="n"/>
-      <c r="L82" s="2" t="n"/>
-      <c r="M82" s="2" t="n"/>
+      <c r="F82" s="2" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>300.4</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>1.075</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>0.694</v>
+      </c>
       <c r="N82" s="2" t="n"/>
       <c r="O82" s="2" t="n">
         <v>7.62</v>
@@ -9264,13 +9360,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.412</v>
+        <v>0.387</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.0016</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -9295,13 +9391,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.58</v>
+        <v>0.576</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
@@ -9326,13 +9422,13 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.32</v>
+        <v>0.336</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0133</v>
+        <v>0.0066</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -9357,13 +9453,13 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.319</v>
+        <v>0.293</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0137</v>
+        <v>0.0187</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -9388,13 +9484,13 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.258</v>
+        <v>0.211</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0487</v>
+        <v>0.0944</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -9419,13 +9515,13 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.346</v>
+        <v>0.351</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0073</v>
+        <v>0.0045</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -9450,13 +9546,13 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.332</v>
+        <v>0.326</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0081</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -9481,17 +9577,17 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.495</v>
+        <v>0.502</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>65</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -9512,13 +9608,13 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.516</v>
+        <v>0.515</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
@@ -9543,13 +9639,13 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.104</v>
+        <v>0.099</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.4312</v>
+        <v>0.4337</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -9574,13 +9670,13 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.301</v>
+        <v>0.277</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0194</v>
+        <v>0.0257</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -9605,13 +9701,13 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.393</v>
+        <v>0.415</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -9636,13 +9732,13 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.39</v>
+        <v>0.382</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0014</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -9667,13 +9763,13 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.505</v>
+        <v>0.518</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
@@ -9698,13 +9794,13 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.571</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -9729,13 +9825,13 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.187</v>
+        <v>0.143</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.1489</v>
+        <v>0.25</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -9760,13 +9856,13 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.387</v>
+        <v>0.357</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0031</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -9791,13 +9887,13 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.517</v>
+        <v>0.532</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
@@ -9822,13 +9918,13 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.212</v>
+        <v>0.2</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.0975</v>
+        <v>0.1017</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -9853,13 +9949,13 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.474</v>
+        <v>0.494</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -9884,13 +9980,13 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.543</v>
+        <v>0.53</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
@@ -9915,13 +10011,13 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>-0.008</v>
+        <v>-0.037</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.9532</v>
+        <v>0.7654</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -9946,13 +10042,13 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.326</v>
+        <v>0.263</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0097</v>
+        <v>0.0304</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -9977,17 +10073,17 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.453</v>
+        <v>0.51</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>68</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -10039,13 +10135,13 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.425</v>
+        <v>0.415</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0028</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -10070,13 +10166,13 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.674</v>
+        <v>0.672</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
@@ -10101,13 +10197,13 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.313</v>
+        <v>0.328</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.0305</v>
+        <v>0.02</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -10132,13 +10228,13 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.258</v>
+        <v>0.256</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0772</v>
+        <v>0.0728</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -10163,13 +10259,13 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.27</v>
+        <v>0.271</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0633</v>
+        <v>0.0567</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -10194,13 +10290,13 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.354</v>
+        <v>0.356</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0136</v>
+        <v>0.0112</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -10225,13 +10321,13 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.417</v>
+        <v>0.413</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0026</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -10256,13 +10352,13 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.569</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
@@ -10287,13 +10383,13 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.542</v>
+        <v>0.554</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
@@ -10318,13 +10414,13 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.177</v>
+        <v>0.173</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.2231</v>
+        <v>0.2247</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -10349,13 +10445,13 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.332</v>
+        <v>0.348</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0198</v>
+        <v>0.0123</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -10380,13 +10476,13 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.414</v>
+        <v>0.429</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0017</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -10411,13 +10507,13 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.473</v>
+        <v>0.475</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.0005</v>
+        <v>0.0004</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -10442,13 +10538,13 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.575</v>
+        <v>0.576</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
@@ -10473,13 +10569,13 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.601</v>
+        <v>0.6</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
@@ -10504,13 +10600,13 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.262</v>
+        <v>0.263</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.0663</v>
+        <v>0.0592</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -10535,13 +10631,13 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.431</v>
+        <v>0.45</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0008</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -10566,13 +10662,13 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.579</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -10597,13 +10693,13 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.233</v>
+        <v>0.245</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.1039</v>
+        <v>0.0806</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -10628,13 +10724,13 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0.513</v>
+        <v>0.524</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>0.0001</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
@@ -10659,13 +10755,13 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0.585</v>
+        <v>0.605</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -10690,13 +10786,13 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>-0.001</v>
+        <v>0.013</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.9926</v>
+        <v>0.9253</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -10721,13 +10817,13 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.356</v>
+        <v>0.359</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.0111</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -10752,13 +10848,13 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.503</v>
+        <v>0.587</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
@@ -10814,17 +10910,17 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0.617</v>
+        <v>0.369</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.0575</v>
+        <v>0.2148</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>13</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -10845,13 +10941,13 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0.149</v>
+        <v>0.338</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.6819</v>
+        <v>0.2593</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -10876,17 +10972,17 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0.487</v>
+        <v>0.504</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.1538</v>
+        <v>0.07870000000000001</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>13</v>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -10907,17 +11003,17 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>0.636</v>
+        <v>0.435</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.0483</v>
+        <v>0.1376</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>13</v>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -10938,13 +11034,13 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>0.476</v>
+        <v>0.152</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.1645</v>
+        <v>0.6209</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -10969,13 +11065,13 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>0.314</v>
+        <v>0.312</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.377</v>
+        <v>0.2998</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -11000,13 +11096,13 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>-0.164</v>
+        <v>-0.129</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.6504</v>
+        <v>0.675</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
@@ -11031,13 +11127,13 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.128</v>
+        <v>0.375</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.7242</v>
+        <v>0.2063</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -11062,13 +11158,13 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.285</v>
+        <v>0.408</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.4243</v>
+        <v>0.1662</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
@@ -11093,13 +11189,13 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>-0.335</v>
+        <v>-0.226</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.3442</v>
+        <v>0.4568</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
@@ -11124,13 +11220,13 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.026</v>
+        <v>-0.05</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.9426</v>
+        <v>0.871</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
@@ -11155,13 +11251,13 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.244</v>
+        <v>0.267</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.4968</v>
+        <v>0.3774</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
@@ -11186,13 +11282,13 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>-0.041</v>
+        <v>-0.047</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.9102</v>
+        <v>0.8721</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
@@ -11217,13 +11313,13 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.121</v>
+        <v>0.45</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.7383999999999999</v>
+        <v>0.1064</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
@@ -11248,13 +11344,13 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.311</v>
+        <v>0.468</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0.3819</v>
+        <v>0.09180000000000001</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
@@ -11279,13 +11375,13 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>-0.195</v>
+        <v>-0.215</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.5893</v>
+        <v>0.4611</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
@@ -11310,13 +11406,13 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0.093</v>
+        <v>0.004</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.7992</v>
+        <v>0.9879</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
@@ -11341,13 +11437,13 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>0.217</v>
+        <v>0.214</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.5461</v>
+        <v>0.4627</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
@@ -11372,13 +11468,13 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.207</v>
+        <v>0.007</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.5407999999999999</v>
+        <v>0.9813</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
@@ -11403,13 +11499,13 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.351</v>
+        <v>0.5</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>0.2897</v>
+        <v>0.0578</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
@@ -11434,13 +11530,13 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.249</v>
+        <v>0.245</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.46</v>
+        <v>0.3778</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
@@ -11465,13 +11561,13 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>0.048</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>0.8888</v>
+        <v>0.8067</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
@@ -11496,13 +11592,13 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0.203</v>
+        <v>-0.029</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.5487</v>
+        <v>0.9181</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
@@ -11527,13 +11623,13 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>0.232</v>
+        <v>0.165</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>0.4932</v>
+        <v>0.5576</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
@@ -11656,17 +11752,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.254</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.0499</v>
+        <v>0.0399</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
@@ -11692,17 +11788,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.247</v>
+        <v>-0.238</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.057</v>
+        <v>0.0548</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
@@ -11728,21 +11824,21 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-0.221</v>
+        <v>-0.182</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.1438</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>66</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -11764,17 +11860,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-0.155</v>
+        <v>0.176</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.2383</v>
+        <v>0.1576</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -11800,17 +11896,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.4947</v>
+        <v>0.5043</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -11836,17 +11932,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-0.063</v>
+        <v>-0.083</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.634</v>
+        <v>0.5062</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -11876,13 +11972,13 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.191</v>
+        <v>0.182</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.1443</v>
+        <v>0.1427</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -11908,17 +12004,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.118</v>
+        <v>-0.125</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.3673</v>
+        <v>0.3192</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -11944,17 +12040,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-0.103</v>
+        <v>-0.124</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.4357</v>
+        <v>0.3221</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -11984,13 +12080,13 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-0.098</v>
+        <v>-0.099</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.4577</v>
+        <v>0.4293</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -12020,13 +12116,13 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.092</v>
+        <v>0.058</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.4851</v>
+        <v>0.6443</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -12056,13 +12152,13 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-0.03</v>
+        <v>-0.029</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.8211000000000001</v>
+        <v>0.8158</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -12308,13 +12404,13 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.365</v>
+        <v>0.366</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.0038</v>
+        <v>0.0023</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
@@ -12340,17 +12436,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>-0.257</v>
+        <v>-0.28</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.0456</v>
+        <v>0.022</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
@@ -12376,17 +12472,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>-0.255</v>
+        <v>-0.276</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.0469</v>
+        <v>0.0238</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
@@ -12416,13 +12512,13 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>-0.226</v>
+        <v>-0.234</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.08</v>
+        <v>0.057</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
@@ -12452,13 +12548,13 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.189</v>
+        <v>0.136</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.1442</v>
+        <v>0.274</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -12488,13 +12584,13 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.033</v>
+        <v>0.029</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.7998</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -12524,17 +12620,17 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.23</v>
+        <v>0.199</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.0751</v>
+        <v>0.1058</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>67</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -12556,17 +12652,17 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>-0.171</v>
+        <v>-0.167</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.187</v>
+        <v>0.1767</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -12592,17 +12688,17 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>-0.166</v>
+        <v>-0.139</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.2014</v>
+        <v>0.2608</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -12632,13 +12728,13 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>-0.138</v>
+        <v>-0.117</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.2885</v>
+        <v>0.3467</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -12668,13 +12764,13 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>-0.102</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.4357</v>
+        <v>0.4814</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -12704,13 +12800,13 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.008</v>
+        <v>-0.021</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.95</v>
+        <v>0.8658</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -12956,13 +13052,13 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.319</v>
+        <v>0.324</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.0116</v>
+        <v>0.007</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
@@ -12992,13 +13088,13 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>-0.248</v>
+        <v>-0.267</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.0519</v>
+        <v>0.0279</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
@@ -13024,17 +13120,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.232</v>
+        <v>-0.249</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.0696</v>
+        <v>0.0408</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
@@ -13060,21 +13156,21 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>-0.224</v>
+        <v>-0.185</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.0794</v>
+        <v>0.13</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>68</v>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13192,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>-0.175</v>
+        <v>0.181</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.1739</v>
+        <v>0.1392</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -13136,13 +13232,13 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.048</v>
+        <v>0.051</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.7135</v>
+        <v>0.6802</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -13168,17 +13264,17 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.243</v>
+        <v>-0.216</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.0572</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
@@ -13204,17 +13300,17 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>-0.221</v>
+        <v>0.204</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.0844</v>
+        <v>0.0958</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
@@ -13244,13 +13340,13 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>-0.204</v>
+        <v>-0.173</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0.1118</v>
+        <v>0.1576</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -13280,13 +13376,13 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>-0.185</v>
+        <v>-0.15</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.149</v>
+        <v>0.2229</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -13316,13 +13412,13 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>-0.142</v>
+        <v>-0.119</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.2701</v>
+        <v>0.3343</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -13352,13 +13448,13 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>-0.023</v>
+        <v>-0.046</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.8604000000000001</v>
+        <v>0.7114</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -13600,21 +13696,21 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.205</v>
+        <v>-0.207</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.1095</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>68</v>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -13636,21 +13732,21 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.196</v>
+        <v>-0.202</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.1268</v>
+        <v>0.0993</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>68</v>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13768,17 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>-0.184</v>
+        <v>0.199</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.1534</v>
+        <v>0.104</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -13708,17 +13804,17 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>-0.171</v>
+        <v>0.155</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.1826</v>
+        <v>0.2065</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -13748,13 +13844,13 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>-0.08500000000000001</v>
+        <v>-0.089</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.5118</v>
+        <v>0.4704</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -13820,13 +13916,13 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>-0.008</v>
+        <v>0.004</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.9538</v>
+        <v>0.9715</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -13892,13 +13988,13 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>-0.181</v>
+        <v>-0.161</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.1593</v>
+        <v>0.1894</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -13924,17 +14020,17 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>-0.171</v>
+        <v>-0.127</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.1835</v>
+        <v>0.3037</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -13960,17 +14056,17 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>-0.161</v>
+        <v>-0.124</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.2108</v>
+        <v>0.3138</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -14000,13 +14096,13 @@
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.148</v>
+        <v>0.097</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.2507</v>
+        <v>0.4307</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -14036,13 +14132,13 @@
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>-0.136</v>
+        <v>-0.09</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.2919</v>
+        <v>0.4665</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -14072,13 +14168,13 @@
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>-0.044</v>
+        <v>-0.083</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.7333</v>
+        <v>0.5031</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -14360,13 +14456,13 @@
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.293</v>
+        <v>0.282</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.0435</v>
+        <v>0.0473</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
@@ -14396,13 +14492,13 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.265</v>
+        <v>0.277</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.0683</v>
+        <v>0.0516</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
@@ -14432,17 +14528,17 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>-0.219</v>
+        <v>-0.248</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>0.1355</v>
+        <v>0.0818</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>50</v>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -14468,13 +14564,13 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>-0.189</v>
+        <v>-0.234</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0.1979</v>
+        <v>0.1014</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -14504,13 +14600,13 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>-0.08799999999999999</v>
+        <v>-0.096</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>0.551</v>
+        <v>0.5084</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -14540,13 +14636,13 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>-0.036</v>
+        <v>-0.06</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>0.8076</v>
+        <v>0.6781</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -14576,13 +14672,13 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.22</v>
+        <v>0.208</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.1322</v>
+        <v>0.1463</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -14612,13 +14708,13 @@
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>-0.106</v>
+        <v>-0.117</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>0.4744</v>
+        <v>0.4166</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -14644,17 +14740,17 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.108</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>0.5422</v>
+        <v>0.4533</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -14680,17 +14776,17 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>-0.08500000000000001</v>
+        <v>-0.098</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0.5667</v>
+        <v>0.4964</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -14720,13 +14816,13 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>0.079</v>
+        <v>0.083</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>0.5948</v>
+        <v>0.5686</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -14756,13 +14852,13 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>-0.042</v>
+        <v>-0.04</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>0.7785</v>
+        <v>0.7819</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -15008,13 +15104,13 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0.39</v>
+        <v>0.415</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.0056</v>
+        <v>0.0025</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
@@ -15044,13 +15140,13 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>-0.312</v>
+        <v>-0.358</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.0288</v>
+        <v>0.0098</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
@@ -15080,13 +15176,13 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>-0.29</v>
+        <v>-0.324</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>0.0436</v>
+        <v>0.0203</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
@@ -15116,17 +15212,17 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>-0.22</v>
+        <v>-0.246</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>0.1292</v>
+        <v>0.0815</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>51</v>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -15152,13 +15248,13 @@
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>0.218</v>
+        <v>0.222</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>0.1319</v>
+        <v>0.118</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -15188,13 +15284,13 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>-0.018</v>
+        <v>-0.042</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>0.904</v>
+        <v>0.7714</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -15224,13 +15320,13 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>0.261</v>
+        <v>0.236</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0956</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
@@ -15256,17 +15352,17 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>-0.203</v>
+        <v>-0.196</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>0.1612</v>
+        <v>0.1689</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -15292,17 +15388,17 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>-0.197</v>
+        <v>-0.178</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>0.1755</v>
+        <v>0.2127</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -15328,17 +15424,17 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>-0.147</v>
+        <v>-0.148</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>0.3149</v>
+        <v>0.299</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -15364,17 +15460,17 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>-0.143</v>
+        <v>-0.131</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>0.3278</v>
+        <v>0.3596</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -15404,13 +15500,13 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>-0.003</v>
+        <v>-0.005</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>0.9853</v>
+        <v>0.9726</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -15656,13 +15752,13 @@
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>0.338</v>
+        <v>0.375</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>0.0164</v>
+        <v>0.0062</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
@@ -15692,13 +15788,13 @@
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>-0.301</v>
+        <v>-0.352</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>0.034</v>
+        <v>0.0105</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H114" s="6" t="inlineStr">
         <is>
@@ -15724,17 +15820,17 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>0.269</v>
+        <v>-0.285</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0.0592</v>
+        <v>0.0402</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
@@ -15760,17 +15856,17 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>-0.244</v>
+        <v>0.271</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>0.0873</v>
+        <v>0.0518</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H116" s="6" t="inlineStr">
         <is>
@@ -15800,13 +15896,13 @@
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>-0.162</v>
+        <v>-0.195</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0.2621</v>
+        <v>0.1662</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -15836,13 +15932,13 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>0.01</v>
+        <v>-0.021</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>0.9474</v>
+        <v>0.8845</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -15872,13 +15968,13 @@
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0.286</v>
+        <v>0.256</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>0.0443</v>
+        <v>0.0664</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H119" s="6" t="inlineStr">
         <is>
@@ -15908,13 +16004,13 @@
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>-0.242</v>
+        <v>-0.24</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>0.091</v>
+        <v>0.0872</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H120" s="6" t="inlineStr">
         <is>
@@ -15944,13 +16040,13 @@
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>-0.219</v>
+        <v>-0.195</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>0.126</v>
+        <v>0.1663</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -15980,13 +16076,13 @@
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>-0.216</v>
+        <v>-0.194</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>0.1325</v>
+        <v>0.1674</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -16016,13 +16112,13 @@
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>-0.163</v>
+        <v>-0.171</v>
       </c>
       <c r="F123" s="2" t="n">
-        <v>0.259</v>
+        <v>0.2262</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -16052,13 +16148,13 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>-0.023</v>
+        <v>-0.025</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>0.872</v>
+        <v>0.8615</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -16300,17 +16396,17 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>0.253</v>
+        <v>-0.324</v>
       </c>
       <c r="F131" s="2" t="n">
-        <v>0.0767</v>
+        <v>0.0193</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
@@ -16336,17 +16432,17 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>-0.252</v>
+        <v>0.311</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>0.077</v>
+        <v>0.0247</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
@@ -16372,17 +16468,17 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>0.248</v>
+        <v>-0.283</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>0.08309999999999999</v>
+        <v>0.0417</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
@@ -16408,21 +16504,21 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>GB%</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>-0.23</v>
+        <v>0.253</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>0.4285</v>
+        <v>0.0704</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="H134" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>52</v>
+      </c>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -16444,17 +16540,17 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>GB%</t>
         </is>
       </c>
       <c r="E135" s="2" t="n">
-        <v>-0.214</v>
+        <v>-0.23</v>
       </c>
       <c r="F135" s="2" t="n">
-        <v>0.1348</v>
+        <v>0.4285</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -16484,13 +16580,13 @@
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>-0.114</v>
+        <v>-0.161</v>
       </c>
       <c r="F136" s="2" t="n">
-        <v>0.4286</v>
+        <v>0.2538</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -16520,13 +16616,13 @@
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>-0.039</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>0.7871</v>
+        <v>0.5495</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -16556,13 +16652,13 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>-0.21</v>
+        <v>-0.194</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>0.1436</v>
+        <v>0.1675</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -16588,17 +16684,17 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E139" s="2" t="n">
-        <v>-0.188</v>
+        <v>-0.165</v>
       </c>
       <c r="F139" s="2" t="n">
-        <v>0.1922</v>
+        <v>0.2414</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -16624,17 +16720,17 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>0.172</v>
+        <v>-0.158</v>
       </c>
       <c r="F140" s="2" t="n">
-        <v>0.2329</v>
+        <v>0.2618</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -16660,17 +16756,17 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>-0.169</v>
+        <v>0.149</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>0.242</v>
+        <v>0.2904</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -16700,13 +16796,13 @@
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>-0.144</v>
+        <v>-0.142</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0.3178</v>
+        <v>0.3137</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -16772,13 +16868,13 @@
         </is>
       </c>
       <c r="E144" s="2" t="n">
-        <v>-0.041</v>
+        <v>-0.059</v>
       </c>
       <c r="F144" s="2" t="n">
-        <v>0.7752</v>
+        <v>0.6762</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -17060,13 +17156,13 @@
         </is>
       </c>
       <c r="E152" s="2" t="n">
-        <v>-0.34</v>
+        <v>-0.285</v>
       </c>
       <c r="F152" s="2" t="n">
-        <v>0.3056</v>
+        <v>0.3037</v>
       </c>
       <c r="G152" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -17092,17 +17188,17 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E153" s="2" t="n">
-        <v>-0.324</v>
+        <v>0.129</v>
       </c>
       <c r="F153" s="2" t="n">
-        <v>0.3316</v>
+        <v>0.6461</v>
       </c>
       <c r="G153" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -17128,17 +17224,17 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E154" s="2" t="n">
-        <v>0.121</v>
+        <v>-0.11</v>
       </c>
       <c r="F154" s="2" t="n">
-        <v>0.7239</v>
+        <v>0.6953</v>
       </c>
       <c r="G154" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -17164,17 +17260,17 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E155" s="2" t="n">
-        <v>-0.114</v>
+        <v>-0.09</v>
       </c>
       <c r="F155" s="2" t="n">
-        <v>0.739</v>
+        <v>0.7499</v>
       </c>
       <c r="G155" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -17204,13 +17300,13 @@
         </is>
       </c>
       <c r="E156" s="2" t="n">
-        <v>-0.058</v>
+        <v>0.065</v>
       </c>
       <c r="F156" s="2" t="n">
-        <v>0.8663</v>
+        <v>0.8166</v>
       </c>
       <c r="G156" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -17236,17 +17332,17 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E157" s="2" t="n">
-        <v>0.007</v>
+        <v>0.061</v>
       </c>
       <c r="F157" s="2" t="n">
-        <v>0.9845</v>
+        <v>0.829</v>
       </c>
       <c r="G157" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -17276,13 +17372,13 @@
         </is>
       </c>
       <c r="E158" s="2" t="n">
-        <v>0.196</v>
+        <v>0.09</v>
       </c>
       <c r="F158" s="2" t="n">
-        <v>0.5636</v>
+        <v>0.7502</v>
       </c>
       <c r="G158" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -17308,17 +17404,17 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E159" s="2" t="n">
-        <v>-0.149</v>
+        <v>0.065</v>
       </c>
       <c r="F159" s="2" t="n">
-        <v>0.6613</v>
+        <v>0.8171</v>
       </c>
       <c r="G159" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -17344,17 +17440,17 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E160" s="2" t="n">
-        <v>-0.119</v>
+        <v>-0.059</v>
       </c>
       <c r="F160" s="2" t="n">
-        <v>0.7275</v>
+        <v>0.8337</v>
       </c>
       <c r="G160" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -17380,17 +17476,17 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E161" s="2" t="n">
-        <v>-0.049</v>
+        <v>-0.016</v>
       </c>
       <c r="F161" s="2" t="n">
-        <v>0.8872</v>
+        <v>0.954</v>
       </c>
       <c r="G161" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -17420,13 +17516,13 @@
         </is>
       </c>
       <c r="E162" s="2" t="n">
-        <v>0.027</v>
+        <v>0.014</v>
       </c>
       <c r="F162" s="2" t="n">
-        <v>0.9374</v>
+        <v>0.9614</v>
       </c>
       <c r="G162" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -17456,13 +17552,13 @@
         </is>
       </c>
       <c r="E163" s="2" t="n">
-        <v>-0.024</v>
+        <v>0.006</v>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.9449</v>
+        <v>0.9829</v>
       </c>
       <c r="G163" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -17492,13 +17588,13 @@
         </is>
       </c>
       <c r="E164" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.499</v>
       </c>
       <c r="F164" s="2" t="n">
-        <v>0.0732</v>
+        <v>0.0586</v>
       </c>
       <c r="G164" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H164" s="6" t="inlineStr">
         <is>
@@ -17528,13 +17624,13 @@
         </is>
       </c>
       <c r="E165" s="2" t="n">
-        <v>-0.331</v>
+        <v>-0.269</v>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.3204</v>
+        <v>0.3319</v>
       </c>
       <c r="G165" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -17560,17 +17656,17 @@
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E166" s="2" t="n">
-        <v>0.158</v>
+        <v>0.153</v>
       </c>
       <c r="F166" s="2" t="n">
-        <v>0.6427</v>
+        <v>0.5856</v>
       </c>
       <c r="G166" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -17596,17 +17692,17 @@
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E167" s="2" t="n">
-        <v>-0.104</v>
+        <v>-0.148</v>
       </c>
       <c r="F167" s="2" t="n">
-        <v>0.761</v>
+        <v>0.5986</v>
       </c>
       <c r="G167" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -17632,17 +17728,17 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E168" s="2" t="n">
-        <v>-0.056</v>
+        <v>0.129</v>
       </c>
       <c r="F168" s="2" t="n">
-        <v>0.8699</v>
+        <v>0.6458</v>
       </c>
       <c r="G168" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -17668,17 +17764,17 @@
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E169" s="2" t="n">
-        <v>0.029</v>
+        <v>0.003</v>
       </c>
       <c r="F169" s="2" t="n">
-        <v>0.9322</v>
+        <v>0.9929</v>
       </c>
       <c r="G169" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -17708,13 +17804,13 @@
         </is>
       </c>
       <c r="E170" s="2" t="n">
-        <v>0.343</v>
+        <v>0.373</v>
       </c>
       <c r="F170" s="2" t="n">
-        <v>0.3012</v>
+        <v>0.1705</v>
       </c>
       <c r="G170" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -17740,17 +17836,17 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E171" s="2" t="n">
-        <v>0.107</v>
+        <v>0.135</v>
       </c>
       <c r="F171" s="2" t="n">
-        <v>0.754</v>
+        <v>0.6318</v>
       </c>
       <c r="G171" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -17776,17 +17872,17 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E172" s="2" t="n">
-        <v>0.081</v>
+        <v>0.096</v>
       </c>
       <c r="F172" s="2" t="n">
-        <v>0.8127</v>
+        <v>0.7345</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -17812,17 +17908,17 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E173" s="2" t="n">
-        <v>0.08</v>
+        <v>-0.052</v>
       </c>
       <c r="F173" s="2" t="n">
-        <v>0.8161</v>
+        <v>0.8549</v>
       </c>
       <c r="G173" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -17848,17 +17944,17 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E174" s="2" t="n">
-        <v>-0.05</v>
+        <v>0.024</v>
       </c>
       <c r="F174" s="2" t="n">
-        <v>0.8829</v>
+        <v>0.9318</v>
       </c>
       <c r="G174" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -17884,17 +17980,17 @@
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E175" s="2" t="n">
-        <v>0.004</v>
+        <v>0.01</v>
       </c>
       <c r="F175" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9707</v>
       </c>
       <c r="G175" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -17924,17 +18020,17 @@
         </is>
       </c>
       <c r="E176" s="2" t="n">
-        <v>0.435</v>
+        <v>0.47</v>
       </c>
       <c r="F176" s="2" t="n">
-        <v>0.1811</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="G176" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="H176" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>15</v>
+      </c>
+      <c r="H176" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -17960,13 +18056,13 @@
         </is>
       </c>
       <c r="E177" s="2" t="n">
-        <v>-0.347</v>
+        <v>-0.278</v>
       </c>
       <c r="F177" s="2" t="n">
-        <v>0.2959</v>
+        <v>0.3149</v>
       </c>
       <c r="G177" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
@@ -17992,17 +18088,17 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E178" s="2" t="n">
-        <v>-0.166</v>
+        <v>-0.169</v>
       </c>
       <c r="F178" s="2" t="n">
-        <v>0.6251</v>
+        <v>0.5468</v>
       </c>
       <c r="G178" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -18032,13 +18128,13 @@
         </is>
       </c>
       <c r="E179" s="2" t="n">
-        <v>0.166</v>
+        <v>0.128</v>
       </c>
       <c r="F179" s="2" t="n">
-        <v>0.6254</v>
+        <v>0.6503</v>
       </c>
       <c r="G179" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -18064,17 +18160,17 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E180" s="2" t="n">
-        <v>-0.08400000000000001</v>
+        <v>0.122</v>
       </c>
       <c r="F180" s="2" t="n">
-        <v>0.806</v>
+        <v>0.664</v>
       </c>
       <c r="G180" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -18100,17 +18196,17 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E181" s="2" t="n">
-        <v>-0.02</v>
+        <v>-0.037</v>
       </c>
       <c r="F181" s="2" t="n">
-        <v>0.9527</v>
+        <v>0.8962</v>
       </c>
       <c r="G181" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -18140,13 +18236,13 @@
         </is>
       </c>
       <c r="E182" s="2" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.206</v>
       </c>
       <c r="F182" s="2" t="n">
-        <v>0.8328</v>
+        <v>0.4617</v>
       </c>
       <c r="G182" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -18172,17 +18268,17 @@
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E183" s="2" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.075</v>
       </c>
       <c r="F183" s="2" t="n">
-        <v>0.8383</v>
+        <v>0.7893</v>
       </c>
       <c r="G183" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -18212,13 +18308,13 @@
         </is>
       </c>
       <c r="E184" s="2" t="n">
-        <v>-0.066</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="F184" s="2" t="n">
-        <v>0.8474</v>
+        <v>0.801</v>
       </c>
       <c r="G184" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -18244,17 +18340,17 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E185" s="2" t="n">
-        <v>-0.065</v>
+        <v>0.036</v>
       </c>
       <c r="F185" s="2" t="n">
-        <v>0.8502999999999999</v>
+        <v>0.8984</v>
       </c>
       <c r="G185" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -18280,17 +18376,17 @@
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E186" s="2" t="n">
-        <v>0.046</v>
+        <v>0.01</v>
       </c>
       <c r="F186" s="2" t="n">
-        <v>0.8925999999999999</v>
+        <v>0.9707</v>
       </c>
       <c r="G186" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -18316,17 +18412,17 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E187" s="2" t="n">
-        <v>-0.015</v>
+        <v>-0</v>
       </c>
       <c r="F187" s="2" t="n">
-        <v>0.9657</v>
+        <v>0.9988</v>
       </c>
       <c r="G187" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -18352,17 +18448,17 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E188" s="2" t="n">
-        <v>0.197</v>
+        <v>0.297</v>
       </c>
       <c r="F188" s="2" t="n">
-        <v>0.5624</v>
+        <v>0.2816</v>
       </c>
       <c r="G188" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -18388,17 +18484,17 @@
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E189" s="2" t="n">
-        <v>0.169</v>
+        <v>-0.25</v>
       </c>
       <c r="F189" s="2" t="n">
-        <v>0.6183999999999999</v>
+        <v>0.3695</v>
       </c>
       <c r="G189" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -18424,17 +18520,17 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E190" s="2" t="n">
-        <v>-0.158</v>
+        <v>0.23</v>
       </c>
       <c r="F190" s="2" t="n">
-        <v>0.6419</v>
+        <v>0.4099</v>
       </c>
       <c r="G190" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -18464,13 +18560,13 @@
         </is>
       </c>
       <c r="E191" s="2" t="n">
-        <v>-0.106</v>
+        <v>-0.195</v>
       </c>
       <c r="F191" s="2" t="n">
-        <v>0.7554999999999999</v>
+        <v>0.485</v>
       </c>
       <c r="G191" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -18496,17 +18592,17 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E192" s="2" t="n">
-        <v>-0.099</v>
+        <v>0.181</v>
       </c>
       <c r="F192" s="2" t="n">
-        <v>0.7714</v>
+        <v>0.5179</v>
       </c>
       <c r="G192" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -18532,17 +18628,17 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E193" s="2" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="F193" s="2" t="n">
-        <v>0.977</v>
+        <v>0.8608</v>
       </c>
       <c r="G193" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -18568,17 +18664,17 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E194" s="2" t="n">
-        <v>-0.21</v>
+        <v>-0.113</v>
       </c>
       <c r="F194" s="2" t="n">
-        <v>0.535</v>
+        <v>0.6877</v>
       </c>
       <c r="G194" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -18604,17 +18700,17 @@
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E195" s="2" t="n">
-        <v>-0.075</v>
+        <v>0.102</v>
       </c>
       <c r="F195" s="2" t="n">
-        <v>0.8274</v>
+        <v>0.7164</v>
       </c>
       <c r="G195" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -18640,17 +18736,17 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E196" s="2" t="n">
-        <v>-0.074</v>
+        <v>-0.063</v>
       </c>
       <c r="F196" s="2" t="n">
-        <v>0.8299</v>
+        <v>0.8222</v>
       </c>
       <c r="G196" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -18676,17 +18772,17 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E197" s="2" t="n">
-        <v>-0.062</v>
+        <v>0.06</v>
       </c>
       <c r="F197" s="2" t="n">
-        <v>0.8561</v>
+        <v>0.8327</v>
       </c>
       <c r="G197" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -18712,17 +18808,17 @@
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E198" s="2" t="n">
-        <v>0.059</v>
+        <v>-0.049</v>
       </c>
       <c r="F198" s="2" t="n">
-        <v>0.8639</v>
+        <v>0.8612</v>
       </c>
       <c r="G198" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -18748,17 +18844,17 @@
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E199" s="2" t="n">
-        <v>-0.053</v>
+        <v>0.027</v>
       </c>
       <c r="F199" s="2" t="n">
-        <v>0.8768</v>
+        <v>0.923</v>
       </c>
       <c r="G199" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -19063,7 +19159,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pitchers with both Asian + MLB data: 62</t>
+          <t>Pitchers with both Asian + MLB data: 68</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Kohei Arihara and Masahide Kobayashi to the correlation sample.
Both had full pre-MLB NPB careers. Arihara's register page had not been linked, and Kobayashi was pointed at a different pitcher.

Co-authored-by: colbymorris08 <colbymorris08@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/asian_pitcher_mlb_analysis.xlsx
+++ b/asian_pitcher_mlb_analysis.xlsx
@@ -6476,14 +6476,30 @@
       <c r="E56" s="2" t="n">
         <v>2008</v>
       </c>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="n"/>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
-      <c r="J56" s="2" t="n"/>
-      <c r="K56" s="2" t="n"/>
-      <c r="L56" s="2" t="n"/>
-      <c r="M56" s="2" t="n"/>
+      <c r="F56" s="2" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>578</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>1.171</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>0.521</v>
+      </c>
       <c r="N56" s="2" t="n"/>
       <c r="O56" s="2" t="n">
         <v>5.1</v>
@@ -7296,14 +7312,30 @@
       <c r="E64" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F64" s="2" t="n"/>
-      <c r="G64" s="2" t="n"/>
-      <c r="H64" s="2" t="n"/>
-      <c r="I64" s="2" t="n"/>
-      <c r="J64" s="2" t="n"/>
-      <c r="K64" s="2" t="n"/>
-      <c r="L64" s="2" t="n"/>
-      <c r="M64" s="2" t="n"/>
+      <c r="F64" s="2" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>834.6</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="J64" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>1.211</v>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="M64" s="2" t="n">
+        <v>0.57</v>
+      </c>
       <c r="N64" s="2" t="n"/>
       <c r="O64" s="2" t="n">
         <v>7.57</v>
@@ -9360,13 +9392,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.387</v>
+        <v>0.394</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0011</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -9391,13 +9423,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.576</v>
+        <v>0.586</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
@@ -9425,10 +9457,10 @@
         <v>0.336</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0066</v>
+        <v>0.0058</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -9453,13 +9485,13 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.293</v>
+        <v>0.289</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0187</v>
+        <v>0.0184</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -9484,13 +9516,13 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.211</v>
+        <v>0.219</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0944</v>
+        <v>0.0775</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -9515,13 +9547,13 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.351</v>
+        <v>0.355</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0045</v>
+        <v>0.0034</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -9546,13 +9578,13 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.326</v>
+        <v>0.319</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.0081</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -9577,13 +9609,13 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.502</v>
+        <v>0.507</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
@@ -9608,13 +9640,13 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.515</v>
+        <v>0.518</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
@@ -9639,13 +9671,13 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.099</v>
+        <v>0.105</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.4337</v>
+        <v>0.3959</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -9670,13 +9702,13 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.277</v>
+        <v>0.261</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0257</v>
+        <v>0.0327</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -9704,10 +9736,10 @@
         <v>0.415</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0005</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -9732,13 +9764,13 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.382</v>
+        <v>0.386</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0014</v>
+        <v>0.0011</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -9763,13 +9795,13 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.518</v>
+        <v>0.526</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
@@ -9794,13 +9826,13 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -9825,13 +9857,13 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.143</v>
+        <v>0.166</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.25</v>
+        <v>0.1734</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -9856,13 +9888,13 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.357</v>
+        <v>0.348</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0034</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -9887,13 +9919,13 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.532</v>
+        <v>0.526</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
@@ -9918,13 +9950,13 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.2</v>
+        <v>0.225</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.1017</v>
+        <v>0.0616</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -9949,17 +9981,17 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.494</v>
+        <v>0.512</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>70</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -9980,13 +10012,13 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.53</v>
+        <v>0.525</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
@@ -10011,13 +10043,13 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>-0.037</v>
+        <v>0.003</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.7654</v>
+        <v>0.9836</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -10042,13 +10074,13 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.263</v>
+        <v>0.265</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0304</v>
+        <v>0.0267</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -10073,13 +10105,13 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.51</v>
+        <v>0.511</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
@@ -10135,13 +10167,13 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.415</v>
+        <v>0.426</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0016</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -10166,13 +10198,13 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.672</v>
+        <v>0.674</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
@@ -10197,13 +10229,13 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.328</v>
+        <v>0.327</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.02</v>
+        <v>0.0179</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -10228,13 +10260,13 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.256</v>
+        <v>0.253</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0728</v>
+        <v>0.0708</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -10259,13 +10291,13 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.271</v>
+        <v>0.283</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0567</v>
+        <v>0.0419</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -10290,13 +10322,13 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.356</v>
+        <v>0.361</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0112</v>
+        <v>0.0086</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -10321,13 +10353,13 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.413</v>
+        <v>0.402</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0028</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -10352,13 +10384,13 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.569</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
@@ -10383,13 +10415,13 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.554</v>
+        <v>0.556</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
@@ -10414,13 +10446,13 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.173</v>
+        <v>0.177</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.2247</v>
+        <v>0.2039</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -10445,13 +10477,13 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.348</v>
+        <v>0.326</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0123</v>
+        <v>0.0173</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -10476,13 +10508,13 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.429</v>
+        <v>0.428</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0014</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -10507,13 +10539,13 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.475</v>
+        <v>0.477</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -10538,13 +10570,13 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.576</v>
+        <v>0.578</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
@@ -10569,13 +10601,13 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.6</v>
+        <v>0.599</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
@@ -10600,13 +10632,13 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.263</v>
+        <v>0.286</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.0592</v>
+        <v>0.0358</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -10631,13 +10663,13 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.45</v>
+        <v>0.434</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0008</v>
+        <v>0.001</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -10662,13 +10694,13 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.579</v>
+        <v>0.57</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -10693,13 +10725,13 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.245</v>
+        <v>0.28</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.0806</v>
+        <v>0.0399</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -10724,13 +10756,13 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0.524</v>
+        <v>0.541</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
@@ -10755,13 +10787,13 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0.605</v>
+        <v>0.597</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -10786,13 +10818,13 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.013</v>
+        <v>0.064</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.9253</v>
+        <v>0.6434</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -10820,10 +10852,10 @@
         <v>0.359</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0076</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -10848,13 +10880,13 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.587</v>
+        <v>0.586</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
@@ -11756,13 +11788,13 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.254</v>
+        <v>0.265</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.0399</v>
+        <v>0.0288</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
@@ -11792,13 +11824,13 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-0.238</v>
+        <v>-0.253</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.0548</v>
+        <v>0.0373</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
@@ -11824,17 +11856,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-0.182</v>
+        <v>0.195</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1438</v>
+        <v>0.1101</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -11860,17 +11892,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.176</v>
+        <v>-0.195</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.1576</v>
+        <v>0.1103</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -11896,17 +11928,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.089</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.5043</v>
+        <v>0.4699</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -11932,17 +11964,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-0.083</v>
+        <v>-0.076</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.5062</v>
+        <v>0.5363</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -11972,13 +12004,13 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.182</v>
+        <v>0.194</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.1427</v>
+        <v>0.1135</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -12008,13 +12040,13 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.125</v>
+        <v>-0.139</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.3192</v>
+        <v>0.2567</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -12044,13 +12076,13 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-0.124</v>
+        <v>-0.137</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.3221</v>
+        <v>0.2649</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -12080,13 +12112,13 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-0.099</v>
+        <v>-0.104</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.4293</v>
+        <v>0.4004</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -12116,13 +12148,13 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.058</v>
+        <v>0.076</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.6443</v>
+        <v>0.5372</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -12152,13 +12184,13 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-0.029</v>
+        <v>-0.025</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.8158</v>
+        <v>0.8404</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -12404,13 +12436,13 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.366</v>
+        <v>0.364</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0021</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
@@ -12443,10 +12475,10 @@
         <v>-0.28</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.022</v>
+        <v>0.0198</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
@@ -12476,13 +12508,13 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>-0.276</v>
+        <v>-0.267</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.0238</v>
+        <v>0.0264</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
@@ -12512,13 +12544,13 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>-0.234</v>
+        <v>-0.213</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.057</v>
+        <v>0.0784</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
@@ -12548,13 +12580,13 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.136</v>
+        <v>0.149</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.274</v>
+        <v>0.2203</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -12584,13 +12616,13 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.029</v>
+        <v>0.02</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.873</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -12620,17 +12652,17 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.199</v>
+        <v>0.2</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.1058</v>
+        <v>0.099</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>69</v>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -12656,13 +12688,13 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>-0.167</v>
+        <v>-0.17</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.1767</v>
+        <v>0.1623</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -12692,13 +12724,13 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>-0.139</v>
+        <v>-0.125</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.2608</v>
+        <v>0.3055</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -12728,13 +12760,13 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>-0.117</v>
+        <v>-0.115</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.3467</v>
+        <v>0.3486</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -12764,13 +12796,13 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.093</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.4814</v>
+        <v>0.4466</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -12800,13 +12832,13 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>-0.021</v>
+        <v>-0.007</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.8658</v>
+        <v>0.955</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -13052,13 +13084,13 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.324</v>
+        <v>0.315</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.007</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
@@ -13088,13 +13120,13 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>-0.267</v>
+        <v>-0.265</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.0279</v>
+        <v>0.0264</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
@@ -13124,13 +13156,13 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>-0.249</v>
+        <v>-0.256</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.0408</v>
+        <v>0.0324</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
@@ -13156,17 +13188,17 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>-0.185</v>
+        <v>0.197</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.13</v>
+        <v>0.1017</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -13192,17 +13224,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.181</v>
+        <v>-0.157</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.1392</v>
+        <v>0.1952</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -13232,13 +13264,13 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.051</v>
+        <v>0.023</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.6802</v>
+        <v>0.8512999999999999</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -13268,13 +13300,13 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>-0.216</v>
+        <v>-0.222</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.07729999999999999</v>
+        <v>0.06469999999999999</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
@@ -13304,13 +13336,13 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.204</v>
+        <v>0.199</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.0958</v>
+        <v>0.0979</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
@@ -13340,13 +13372,13 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>-0.173</v>
+        <v>-0.175</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0.1576</v>
+        <v>0.1463</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -13372,17 +13404,17 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.137</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.2229</v>
+        <v>0.2598</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -13408,17 +13440,17 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>-0.119</v>
+        <v>-0.129</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.3343</v>
+        <v>0.2883</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -13448,13 +13480,13 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>-0.046</v>
+        <v>-0.028</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.7114</v>
+        <v>0.8153</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -13700,13 +13732,13 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>-0.207</v>
+        <v>-0.22</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.0678</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
@@ -13732,17 +13764,17 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>-0.202</v>
+        <v>0.206</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.0993</v>
+        <v>0.0876</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
@@ -13768,21 +13800,21 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.199</v>
+        <v>-0.205</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.104</v>
+        <v>0.089</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>70</v>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -13808,13 +13840,13 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.155</v>
+        <v>0.182</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.2065</v>
+        <v>0.1321</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -13844,13 +13876,13 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>-0.089</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.4704</v>
+        <v>0.5604</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -13916,13 +13948,13 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.004</v>
+        <v>-0.016</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.9715</v>
+        <v>0.8959</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -13988,13 +14020,13 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>-0.161</v>
+        <v>-0.17</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.1894</v>
+        <v>0.1584</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -14020,17 +14052,17 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>-0.127</v>
+        <v>-0.128</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.3037</v>
+        <v>0.2918</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -14056,17 +14088,17 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>-0.124</v>
+        <v>-0.113</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.3138</v>
+        <v>0.3506</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -14096,13 +14128,13 @@
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.097</v>
+        <v>0.105</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.4307</v>
+        <v>0.3874</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -14132,13 +14164,13 @@
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.101</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.4665</v>
+        <v>0.4065</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -14168,13 +14200,13 @@
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>-0.083</v>
+        <v>-0.057</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.5031</v>
+        <v>0.6408</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -14456,13 +14488,13 @@
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.282</v>
+        <v>0.301</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.0473</v>
+        <v>0.0304</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
@@ -14492,13 +14524,13 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.277</v>
+        <v>0.291</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.0516</v>
+        <v>0.0366</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
@@ -14528,13 +14560,13 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>-0.248</v>
+        <v>-0.276</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>0.0818</v>
+        <v>0.0475</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
@@ -14564,17 +14596,17 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>-0.234</v>
+        <v>-0.255</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0.1014</v>
+        <v>0.0684</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>52</v>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -14600,13 +14632,13 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>-0.096</v>
+        <v>-0.104</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>0.5084</v>
+        <v>0.4624</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -14636,13 +14668,13 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>-0.06</v>
+        <v>-0.051</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>0.6781</v>
+        <v>0.7176</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -14672,13 +14704,13 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.208</v>
+        <v>0.223</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.1463</v>
+        <v>0.1126</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -14704,17 +14736,17 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>-0.117</v>
+        <v>-0.136</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>0.4166</v>
+        <v>0.3367</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -14740,17 +14772,17 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>-0.108</v>
+        <v>-0.124</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>0.4533</v>
+        <v>0.3799</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -14780,13 +14812,13 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>-0.098</v>
+        <v>-0.121</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0.4964</v>
+        <v>0.3909</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -14816,13 +14848,13 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>0.083</v>
+        <v>0.104</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>0.5686</v>
+        <v>0.4627</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -14852,13 +14884,13 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>-0.04</v>
+        <v>-0.034</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>0.7819</v>
+        <v>0.8097</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -15104,13 +15136,13 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0.415</v>
+        <v>0.408</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0024</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
@@ -15140,13 +15172,13 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>-0.358</v>
+        <v>-0.347</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.0098</v>
+        <v>0.011</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
@@ -15176,13 +15208,13 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>-0.324</v>
+        <v>-0.326</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>0.0203</v>
+        <v>0.0171</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
@@ -15208,17 +15240,17 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>-0.246</v>
+        <v>0.234</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>0.0815</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
@@ -15244,17 +15276,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>0.222</v>
+        <v>-0.219</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>0.118</v>
+        <v>0.1158</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -15284,13 +15316,13 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>-0.042</v>
+        <v>-0.051</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>0.7714</v>
+        <v>0.7159</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -15323,10 +15355,10 @@
         <v>0.236</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>0.0956</v>
+        <v>0.0893</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
@@ -15356,13 +15388,13 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>-0.196</v>
+        <v>-0.202</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>0.1689</v>
+        <v>0.1479</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -15392,13 +15424,13 @@
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>-0.178</v>
+        <v>-0.157</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>0.2127</v>
+        <v>0.2607</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -15428,13 +15460,13 @@
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>-0.148</v>
+        <v>-0.154</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>0.299</v>
+        <v>0.2711</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -15464,13 +15496,13 @@
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>-0.131</v>
+        <v>-0.13</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>0.3596</v>
+        <v>0.3545</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -15500,13 +15532,13 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>-0.005</v>
+        <v>0.011</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>0.9726</v>
+        <v>0.9379</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -15752,13 +15784,13 @@
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>0.375</v>
+        <v>0.36</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>0.0062</v>
+        <v>0.0075</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
@@ -15788,13 +15820,13 @@
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>-0.352</v>
+        <v>-0.349</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>0.0105</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H114" s="6" t="inlineStr">
         <is>
@@ -15824,13 +15856,13 @@
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>-0.285</v>
+        <v>-0.296</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0.0402</v>
+        <v>0.0298</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
@@ -15860,13 +15892,13 @@
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0.271</v>
+        <v>0.286</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>0.0518</v>
+        <v>0.036</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H116" s="6" t="inlineStr">
         <is>
@@ -15896,13 +15928,13 @@
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>-0.195</v>
+        <v>-0.156</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0.1662</v>
+        <v>0.2595</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -15932,13 +15964,13 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>-0.021</v>
+        <v>-0.052</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>0.8845</v>
+        <v>0.7113</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -15964,17 +15996,17 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0.256</v>
+        <v>-0.249</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>0.0664</v>
+        <v>0.06909999999999999</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H119" s="6" t="inlineStr">
         <is>
@@ -16000,17 +16032,17 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>-0.24</v>
+        <v>0.249</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>0.0872</v>
+        <v>0.0696</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H120" s="6" t="inlineStr">
         <is>
@@ -16036,17 +16068,17 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>-0.195</v>
+        <v>-0.198</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>0.1663</v>
+        <v>0.1502</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -16072,17 +16104,17 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>-0.194</v>
+        <v>-0.191</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>0.1674</v>
+        <v>0.1667</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -16108,17 +16140,17 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>-0.171</v>
+        <v>-0.165</v>
       </c>
       <c r="F123" s="2" t="n">
-        <v>0.2262</v>
+        <v>0.2336</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -16148,13 +16180,13 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.005</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>0.8615</v>
+        <v>0.9736</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -16400,13 +16432,13 @@
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>-0.324</v>
+        <v>-0.326</v>
       </c>
       <c r="F131" s="2" t="n">
-        <v>0.0193</v>
+        <v>0.016</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
@@ -16436,13 +16468,13 @@
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>0.311</v>
+        <v>0.314</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>0.0247</v>
+        <v>0.0207</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
@@ -16472,13 +16504,13 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>-0.283</v>
+        <v>-0.302</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>0.0417</v>
+        <v>0.0263</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
@@ -16508,13 +16540,13 @@
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>0.253</v>
+        <v>0.281</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>0.0704</v>
+        <v>0.0398</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H134" s="6" t="inlineStr">
         <is>
@@ -16580,13 +16612,13 @@
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>-0.161</v>
+        <v>-0.133</v>
       </c>
       <c r="F136" s="2" t="n">
-        <v>0.2538</v>
+        <v>0.3365</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -16616,13 +16648,13 @@
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>-0.08500000000000001</v>
+        <v>-0.106</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>0.5495</v>
+        <v>0.4457</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -16652,13 +16684,13 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>-0.194</v>
+        <v>-0.21</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>0.1675</v>
+        <v>0.1278</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -16684,17 +16716,17 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E139" s="2" t="n">
         <v>-0.165</v>
       </c>
       <c r="F139" s="2" t="n">
-        <v>0.2414</v>
+        <v>0.234</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -16720,17 +16752,17 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>-0.158</v>
+        <v>0.157</v>
       </c>
       <c r="F140" s="2" t="n">
-        <v>0.2618</v>
+        <v>0.2571</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -16756,17 +16788,17 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>0.149</v>
+        <v>-0.154</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>0.2904</v>
+        <v>0.2654</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -16792,17 +16824,17 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>-0.142</v>
+        <v>-0.145</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0.3137</v>
+        <v>0.2947</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -16868,13 +16900,13 @@
         </is>
       </c>
       <c r="E144" s="2" t="n">
-        <v>-0.059</v>
+        <v>-0.028</v>
       </c>
       <c r="F144" s="2" t="n">
-        <v>0.6762</v>
+        <v>0.8406</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -19159,7 +19191,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pitchers with both Asian + MLB data: 68</t>
+          <t>Pitchers with both Asian + MLB data: 70</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the pre-MLB Asian careers missing from the roster.
Shohei Ohtani, Tomo Ohka, and the other verified NPB and KBO arrivals now sit in the all-pitchers table. Fukumori and Lim stay out of the correlations because their MLB samples are under 10 innings.

Co-authored-by: colbymorris08 <colbymorris08@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/asian_pitcher_mlb_analysis.xlsx
+++ b/asian_pitcher_mlb_analysis.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG82"/>
+  <dimension ref="A1:AG96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -9315,6 +9315,1490 @@
         <v>0</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Takashi Kashiwada</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>1997</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>1.517</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="N83" s="2" t="n"/>
+      <c r="O83" s="2" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="P83" s="2" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="Q83" s="2" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="R83" s="2" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="S83" s="2" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="T83" s="2" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="U83" s="2" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="V83" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="W83" s="2" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="X83" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="Y83" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Z83" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA83" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB83" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC83" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE83" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="AF83" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="AG83" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Masao Kida</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>1999</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>971.5</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="J84" s="2" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="K84" s="2" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="N84" s="2" t="n"/>
+      <c r="O84" s="2" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="P84" s="2" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="Q84" s="2" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="R84" s="2" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="S84" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="T84" s="2" t="n">
+        <v>1.607</v>
+      </c>
+      <c r="U84" s="2" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="V84" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W84" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="X84" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="Y84" s="2" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="Z84" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA84" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB84" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC84" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="AD84" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE84" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="AF84" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="AG84" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Tomo Ohka</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>1999</v>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="J85" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K85" s="2" t="n">
+        <v>1.887</v>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="M85" s="2" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="N85" s="2" t="n"/>
+      <c r="O85" s="2" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="P85" s="2" t="n">
+        <v>1070</v>
+      </c>
+      <c r="Q85" s="2" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="R85" s="2" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="S85" s="2" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="T85" s="2" t="n">
+        <v>1.387</v>
+      </c>
+      <c r="U85" s="2" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="V85" s="2" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="W85" s="2" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="X85" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="Y85" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z85" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA85" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="AB85" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="AC85" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="AD85" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="AE85" s="2" t="n">
+        <v>590</v>
+      </c>
+      <c r="AF85" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="AG85" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Takahito Nomura</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>2002</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>423.2</v>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>10.06</v>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="J86" s="2" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="K86" s="2" t="n">
+        <v>1.281</v>
+      </c>
+      <c r="L86" s="2" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="M86" s="2" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="N86" s="2" t="n"/>
+      <c r="O86" s="2" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="P86" s="2" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="Q86" s="2" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="R86" s="2" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="S86" s="2" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="T86" s="2" t="n">
+        <v>2.197</v>
+      </c>
+      <c r="U86" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V86" s="2" t="n"/>
+      <c r="W86" s="2" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="X86" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="Y86" s="2" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="Z86" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC86" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="AD86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE86" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AF86" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="AG86" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Kazuo Fukumori</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>2008</v>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>658.9</v>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="I87" s="2" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="J87" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="K87" s="2" t="n">
+        <v>1.383</v>
+      </c>
+      <c r="L87" s="2" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="M87" s="2" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="N87" s="2" t="n"/>
+      <c r="O87" s="2" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="P87" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q87" s="2" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="R87" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="S87" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="T87" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="U87" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="V87" s="2" t="n"/>
+      <c r="W87" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="X87" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="Y87" s="2" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="Z87" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC87" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE87" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF87" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG87" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Yasuhiko Yabuta</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>2008</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>827.3</v>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J88" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="K88" s="2" t="n">
+        <v>1.355</v>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="M88" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N88" s="2" t="n"/>
+      <c r="O88" s="2" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="P88" s="2" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="Q88" s="2" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="R88" s="2" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="S88" s="2" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="T88" s="2" t="n">
+        <v>1.836</v>
+      </c>
+      <c r="U88" s="2" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="V88" s="2" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="W88" s="2" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="X88" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="Y88" s="2" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="Z88" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA88" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB88" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC88" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="AD88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE88" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="AF88" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="AG88" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Ken Takahashi</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>2009</v>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="G89" s="2" t="n">
+        <v>1427.8</v>
+      </c>
+      <c r="H89" s="2" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="I89" s="2" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="J89" s="2" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="K89" s="2" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="L89" s="2" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="M89" s="2" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="N89" s="2" t="n"/>
+      <c r="O89" s="2" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="P89" s="2" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="Q89" s="2" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="R89" s="2" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="S89" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="T89" s="2" t="n">
+        <v>1.365</v>
+      </c>
+      <c r="U89" s="2" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="V89" s="2" t="n"/>
+      <c r="W89" s="2" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="X89" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="Y89" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="Z89" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB89" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC89" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE89" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="AF89" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="AG89" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Yoshinori Tateyama</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>659.8</v>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="J90" s="2" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="K90" s="2" t="n">
+        <v>1.167</v>
+      </c>
+      <c r="L90" s="2" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="M90" s="2" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="N90" s="2" t="n"/>
+      <c r="O90" s="2" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="P90" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="Q90" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="R90" s="2" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="S90" s="2" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="T90" s="2" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="U90" s="2" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="V90" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W90" s="2" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="X90" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="Y90" s="2" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="Z90" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA90" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC90" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="AD90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE90" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="AF90" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="AG90" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="G91" s="2" t="n">
+        <v>541.6</v>
+      </c>
+      <c r="H91" s="2" t="n">
+        <v>10.37</v>
+      </c>
+      <c r="I91" s="2" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="J91" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K91" s="2" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="M91" s="2" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="N91" s="2" t="n"/>
+      <c r="O91" s="2" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="P91" s="2" t="n">
+        <v>614.1</v>
+      </c>
+      <c r="Q91" s="2" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="R91" s="2" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="S91" s="2" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="T91" s="2" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="U91" s="2" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="V91" s="2" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="W91" s="2" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="X91" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="Y91" s="2" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="Z91" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA91" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="AB91" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="AC91" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="AD91" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="AE91" s="2" t="n">
+        <v>765</v>
+      </c>
+      <c r="AF91" s="2" t="n">
+        <v>208</v>
+      </c>
+      <c r="AG91" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Sang-Hoon Lee</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="G92" s="2" t="n">
+        <v>879</v>
+      </c>
+      <c r="H92" s="2" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="I92" s="2" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="J92" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K92" s="2" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="M92" s="2" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="N92" s="2" t="n"/>
+      <c r="O92" s="2" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="P92" s="2" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="Q92" s="2" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="R92" s="2" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="S92" s="2" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="T92" s="2" t="n">
+        <v>1.339</v>
+      </c>
+      <c r="U92" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="V92" s="2" t="n"/>
+      <c r="W92" s="2" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="X92" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="Y92" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z92" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC92" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AD92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE92" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF92" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG92" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Dae-Sung Koo</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>2005</v>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="G93" s="2" t="n">
+        <v>1415.3</v>
+      </c>
+      <c r="H93" s="2" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="I93" s="2" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J93" s="2" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="K93" s="2" t="n">
+        <v>1.188</v>
+      </c>
+      <c r="L93" s="2" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="M93" s="2" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="N93" s="2" t="n"/>
+      <c r="O93" s="2" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="P93" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q93" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="R93" s="2" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="S93" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="T93" s="2" t="n">
+        <v>1.522</v>
+      </c>
+      <c r="U93" s="2" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="V93" s="2" t="n"/>
+      <c r="W93" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="X93" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="Y93" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Z93" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC93" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="AD93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE93" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="AF93" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="AG93" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Chang-Yong Lim</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="n">
+        <v>2013</v>
+      </c>
+      <c r="F94" s="2" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G94" s="2" t="n">
+        <v>1682.7</v>
+      </c>
+      <c r="H94" s="2" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="I94" s="2" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="J94" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="K94" s="2" t="n">
+        <v>1.129</v>
+      </c>
+      <c r="L94" s="2" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="M94" s="2" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="N94" s="2" t="n"/>
+      <c r="O94" s="2" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="P94" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q94" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="R94" s="2" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="S94" s="2" t="n"/>
+      <c r="T94" s="2" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="U94" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="V94" s="2" t="n"/>
+      <c r="W94" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="X94" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="Y94" s="2" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Z94" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC94" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE94" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF94" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG94" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Yariel Rodriguez</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F95" s="2" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="G95" s="2" t="n">
+        <v>174.4</v>
+      </c>
+      <c r="H95" s="2" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="I95" s="2" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="J95" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="K95" s="2" t="n">
+        <v>1.233</v>
+      </c>
+      <c r="L95" s="2" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="M95" s="2" t="n">
+        <v>0.554</v>
+      </c>
+      <c r="N95" s="2" t="n"/>
+      <c r="O95" s="2" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="P95" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="Q95" s="2" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="R95" s="2" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="S95" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="T95" s="2" t="n">
+        <v>1.284</v>
+      </c>
+      <c r="U95" s="2" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="V95" s="2" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="W95" s="2" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="X95" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="Y95" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z95" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA95" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB95" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC95" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="AD95" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="AE95" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="AF95" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="AG95" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Reed Garrett</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="G96" s="2" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>8.81</v>
+      </c>
+      <c r="I96" s="2" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="J96" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="K96" s="2" t="n">
+        <v>1.525</v>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="M96" s="2" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="N96" s="2" t="n"/>
+      <c r="O96" s="2" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="P96" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="Q96" s="2" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="R96" s="2" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="S96" s="2" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="T96" s="2" t="n">
+        <v>1.529</v>
+      </c>
+      <c r="U96" s="2" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="V96" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W96" s="2" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="X96" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="Y96" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Z96" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA96" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB96" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC96" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="AD96" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE96" s="2" t="n">
+        <v>179</v>
+      </c>
+      <c r="AF96" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="AG96" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9392,13 +10876,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.394</v>
+        <v>0.414</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0002</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -9423,13 +10907,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.586</v>
+        <v>0.609</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
@@ -9454,13 +10938,13 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.336</v>
+        <v>0.313</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0058</v>
+        <v>0.0062</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -9485,13 +10969,13 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.289</v>
+        <v>0.224</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0184</v>
+        <v>0.0529</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -9516,13 +11000,13 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.219</v>
+        <v>0.33</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0775</v>
+        <v>0.0038</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -9547,13 +11031,13 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.355</v>
+        <v>0.409</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0034</v>
+        <v>0.0003</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -9578,13 +11062,13 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.319</v>
+        <v>0.356</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0014</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -9609,13 +11093,13 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.507</v>
+        <v>0.544</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
@@ -9640,17 +11124,17 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.518</v>
+        <v>0.485</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>78</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -9671,13 +11155,13 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.105</v>
+        <v>0.037</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.3959</v>
+        <v>0.7485000000000001</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -9702,13 +11186,13 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.261</v>
+        <v>0.392</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0327</v>
+        <v>0.0004</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -9733,13 +11217,13 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.415</v>
+        <v>0.47</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -9764,13 +11248,13 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.386</v>
+        <v>0.319</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0037</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -9795,13 +11279,13 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.526</v>
+        <v>0.544</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
@@ -9826,17 +11310,17 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.422</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>81</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -9857,13 +11341,13 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.166</v>
+        <v>0.067</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.1734</v>
+        <v>0.5548</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -9888,13 +11372,13 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.348</v>
+        <v>0.374</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0034</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -9919,13 +11403,13 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.526</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
@@ -9950,13 +11434,13 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.225</v>
+        <v>0.212</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.0616</v>
+        <v>0.0555</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -9981,13 +11465,13 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.512</v>
+        <v>0.54</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
@@ -10012,17 +11496,17 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.525</v>
+        <v>0.386</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>82</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -10043,13 +11527,13 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.003</v>
+        <v>-0.034</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.9836</v>
+        <v>0.7651</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -10074,13 +11558,13 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.265</v>
+        <v>0.306</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0267</v>
+        <v>0.0051</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -10105,13 +11589,13 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.511</v>
+        <v>0.539</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
@@ -10167,13 +11651,13 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.426</v>
+        <v>0.447</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0003</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -10198,13 +11682,13 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.674</v>
+        <v>0.6860000000000001</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
@@ -10229,13 +11713,13 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.327</v>
+        <v>0.301</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.0179</v>
+        <v>0.0183</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -10260,13 +11744,13 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.253</v>
+        <v>0.18</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0708</v>
+        <v>0.1652</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -10291,13 +11775,13 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.283</v>
+        <v>0.415</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0419</v>
+        <v>0.0009</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -10322,13 +11806,13 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.361</v>
+        <v>0.421</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0086</v>
+        <v>0.0007</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -10353,13 +11837,13 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.402</v>
+        <v>0.43</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0004</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -10384,13 +11868,13 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.594</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
@@ -10415,17 +11899,17 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.556</v>
+        <v>0.5</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>64</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -10446,13 +11930,13 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.177</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.2039</v>
+        <v>0.5095</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -10477,13 +11961,13 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.326</v>
+        <v>0.467</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0173</v>
+        <v>0.0001</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -10508,13 +11992,13 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.428</v>
+        <v>0.489</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.0014</v>
+        <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -10539,13 +12023,13 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.477</v>
+        <v>0.373</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.0003</v>
+        <v>0.002</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -10570,13 +12054,13 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.578</v>
+        <v>0.589</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
@@ -10601,17 +12085,17 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.599</v>
+        <v>0.425</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>66</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -10632,13 +12116,13 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.286</v>
+        <v>0.153</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.0358</v>
+        <v>0.2203</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -10663,13 +12147,13 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.434</v>
+        <v>0.44</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0002</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -10694,13 +12178,13 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.57</v>
+        <v>0.604</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -10725,13 +12209,13 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.28</v>
+        <v>0.256</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.0399</v>
+        <v>0.0381</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -10756,13 +12240,13 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0.541</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
@@ -10787,17 +12271,17 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0.597</v>
+        <v>0.405</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>0.0007</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>66</v>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -10818,13 +12302,13 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.064</v>
+        <v>0.016</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.6434</v>
+        <v>0.8984</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -10849,13 +12333,13 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.359</v>
+        <v>0.382</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.0076</v>
+        <v>0.0015</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -10880,13 +12364,13 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.586</v>
+        <v>0.608</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
@@ -11784,17 +13268,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.265</v>
+        <v>-0.25</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.0288</v>
+        <v>0.0273</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
@@ -11820,17 +13304,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-0.253</v>
+        <v>-0.212</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.0373</v>
+        <v>0.0624</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
@@ -11856,21 +13340,21 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.195</v>
+        <v>0.203</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1101</v>
+        <v>0.0745</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>78</v>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -11892,17 +13376,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-0.195</v>
+        <v>0.155</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.1103</v>
+        <v>0.1766</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -11932,13 +13416,13 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-0.089</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.4699</v>
+        <v>0.4517</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -11968,13 +13452,13 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-0.076</v>
+        <v>-0.022</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.5363</v>
+        <v>0.8473000000000001</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -12004,17 +13488,17 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.194</v>
+        <v>0.197</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.1135</v>
+        <v>0.0834</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>78</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -12036,17 +13520,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.139</v>
+        <v>-0.171</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.2567</v>
+        <v>0.1346</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -12072,17 +13556,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-0.137</v>
+        <v>-0.164</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.2649</v>
+        <v>0.1526</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -12108,17 +13592,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-0.104</v>
+        <v>0.148</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.4004</v>
+        <v>0.1956</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -12144,17 +13628,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.076</v>
+        <v>-0.134</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.5372</v>
+        <v>0.2415</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -12184,13 +13668,13 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-0.025</v>
+        <v>0.025</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.8404</v>
+        <v>0.8250999999999999</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -12436,13 +13920,13 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.364</v>
+        <v>0.325</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0033</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
@@ -12468,17 +13952,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.281</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.0198</v>
+        <v>0.0115</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
@@ -12504,17 +13988,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>-0.267</v>
+        <v>-0.277</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.0264</v>
+        <v>0.0127</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
@@ -12544,13 +14028,13 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>-0.213</v>
+        <v>-0.197</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.0784</v>
+        <v>0.07969999999999999</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
@@ -12580,13 +14064,13 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.149</v>
+        <v>0.123</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.2203</v>
+        <v>0.2787</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -12616,13 +14100,13 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.873</v>
+        <v>0.9284</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -12652,13 +14136,13 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.2</v>
+        <v>0.243</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.099</v>
+        <v>0.0297</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
@@ -12688,17 +14172,17 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>-0.17</v>
+        <v>-0.217</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.1623</v>
+        <v>0.0535</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>80</v>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -12720,21 +14204,21 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>-0.125</v>
+        <v>-0.198</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.3055</v>
+        <v>0.0776</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>80</v>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -12756,17 +14240,17 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>-0.115</v>
+        <v>-0.163</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.3486</v>
+        <v>0.1494</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -12796,13 +14280,13 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>-0.093</v>
+        <v>-0.156</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.4466</v>
+        <v>0.1684</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -12832,13 +14316,13 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>-0.007</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.955</v>
+        <v>0.4613</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -13084,13 +14568,13 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.315</v>
+        <v>0.284</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0098</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
@@ -13120,13 +14604,13 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>-0.265</v>
+        <v>-0.238</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.0264</v>
+        <v>0.0311</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
@@ -13156,13 +14640,13 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>-0.256</v>
+        <v>-0.214</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.0324</v>
+        <v>0.053</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
@@ -13192,13 +14676,13 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.197</v>
+        <v>0.182</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.1017</v>
+        <v>0.1023</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -13228,13 +14712,13 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>-0.157</v>
+        <v>-0.134</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.1952</v>
+        <v>0.2294</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -13264,13 +14748,13 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.023</v>
+        <v>-0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.8512999999999999</v>
+        <v>0.9989</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -13296,17 +14780,17 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>-0.222</v>
+        <v>0.214</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.0536</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
@@ -13332,21 +14816,21 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.199</v>
+        <v>-0.167</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.0979</v>
+        <v>0.1347</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>82</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -13372,13 +14856,13 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>-0.175</v>
+        <v>-0.142</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0.1463</v>
+        <v>0.2016</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -13404,17 +14888,17 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>-0.137</v>
+        <v>-0.135</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.2598</v>
+        <v>0.2277</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -13444,13 +14928,13 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>-0.129</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.2883</v>
+        <v>0.4332</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -13480,13 +14964,13 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>-0.028</v>
+        <v>0.029</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.8153</v>
+        <v>0.7972</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -13732,13 +15216,13 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>-0.22</v>
+        <v>-0.222</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.0678</v>
+        <v>0.0446</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
@@ -13764,17 +15248,17 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.206</v>
+        <v>-0.218</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.0876</v>
+        <v>0.0489</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
@@ -13800,17 +15284,17 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>-0.205</v>
+        <v>0.198</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.089</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
@@ -13840,13 +15324,13 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.182</v>
+        <v>0.161</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.1321</v>
+        <v>0.1489</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -13876,13 +15360,13 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.081</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.5604</v>
+        <v>0.4701</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -13908,17 +15392,17 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>GB%</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
         <v>-0.047</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.854</v>
+        <v>0.6762</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -13944,17 +15428,17 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>GB%</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>-0.016</v>
+        <v>-0.047</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.8959</v>
+        <v>0.854</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -14016,21 +15500,21 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>-0.17</v>
+        <v>-0.193</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.1584</v>
+        <v>0.0829</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>82</v>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -14052,17 +15536,17 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>-0.128</v>
+        <v>-0.163</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.2918</v>
+        <v>0.1428</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -14088,17 +15572,17 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>-0.113</v>
+        <v>0.131</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.3506</v>
+        <v>0.2404</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -14124,17 +15608,17 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.105</v>
+        <v>-0.121</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.3874</v>
+        <v>0.279</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -14160,17 +15644,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>-0.101</v>
+        <v>-0.065</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.4065</v>
+        <v>0.5637</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -14200,13 +15684,13 @@
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>-0.057</v>
+        <v>0.006</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.6408</v>
+        <v>0.9585</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -14484,17 +15968,17 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.301</v>
+        <v>-0.274</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.0304</v>
+        <v>0.0315</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
@@ -14520,17 +16004,17 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.291</v>
+        <v>-0.27</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.0366</v>
+        <v>0.0338</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
@@ -14556,17 +16040,17 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>-0.276</v>
+        <v>0.232</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>0.0475</v>
+        <v>0.0696</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
@@ -14592,17 +16076,17 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>-0.255</v>
+        <v>0.221</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0.0684</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
@@ -14632,13 +16116,13 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>-0.104</v>
+        <v>-0.103</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>0.4624</v>
+        <v>0.4242</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -14668,13 +16152,13 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>-0.051</v>
+        <v>-0.005</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>0.7176</v>
+        <v>0.9673</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -14704,17 +16188,17 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.223</v>
+        <v>0.23</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.1126</v>
+        <v>0.0725</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>62</v>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -14736,17 +16220,17 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>-0.136</v>
+        <v>0.185</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>0.3367</v>
+        <v>0.1504</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -14772,17 +16256,17 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>-0.124</v>
+        <v>-0.18</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>0.3799</v>
+        <v>0.1608</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -14812,13 +16296,13 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>-0.121</v>
+        <v>-0.177</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0.3909</v>
+        <v>0.1679</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -14844,17 +16328,17 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>0.104</v>
+        <v>-0.163</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>0.4627</v>
+        <v>0.2058</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -14884,13 +16368,13 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>-0.034</v>
+        <v>0.016</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>0.8097</v>
+        <v>0.9006999999999999</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -15136,13 +16620,13 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0.408</v>
+        <v>0.364</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0031</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
@@ -15172,13 +16656,13 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>-0.347</v>
+        <v>-0.353</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.011</v>
+        <v>0.0042</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
@@ -15208,13 +16692,13 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>-0.326</v>
+        <v>-0.318</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>0.0171</v>
+        <v>0.0103</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
@@ -15240,17 +16724,17 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>0.234</v>
+        <v>-0.208</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>0.09229999999999999</v>
+        <v>0.0998</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
@@ -15276,17 +16760,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>-0.219</v>
+        <v>0.187</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>0.1158</v>
+        <v>0.1399</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -15316,13 +16800,13 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>-0.051</v>
+        <v>-0.047</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>0.7159</v>
+        <v>0.7119</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -15352,13 +16836,13 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>0.236</v>
+        <v>0.285</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>0.0893</v>
+        <v>0.0223</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
@@ -15388,17 +16872,17 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>-0.202</v>
+        <v>-0.258</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>0.1479</v>
+        <v>0.0397</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="H102" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>64</v>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -15420,21 +16904,21 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>-0.157</v>
+        <v>-0.234</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>0.2607</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="H103" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>64</v>
+      </c>
+      <c r="H103" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -15460,17 +16944,17 @@
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>-0.154</v>
+        <v>-0.213</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>0.2711</v>
+        <v>0.0916</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="H104" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>64</v>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -15492,17 +16976,17 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>-0.13</v>
+        <v>-0.201</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>0.3545</v>
+        <v>0.1118</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -15532,13 +17016,13 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>0.011</v>
+        <v>0.112</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>0.9379</v>
+        <v>0.3772</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -15784,13 +17268,13 @@
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>0.36</v>
+        <v>0.324</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>0.0075</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
@@ -15820,13 +17304,13 @@
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>-0.349</v>
+        <v>-0.298</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.015</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H114" s="6" t="inlineStr">
         <is>
@@ -15852,17 +17336,17 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/9</t>
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>-0.296</v>
+        <v>0.255</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0.0298</v>
+        <v>0.0388</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
@@ -15888,17 +17372,17 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>K/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0.286</v>
+        <v>-0.242</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>0.036</v>
+        <v>0.0503</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H116" s="6" t="inlineStr">
         <is>
@@ -15928,13 +17412,13 @@
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>-0.156</v>
+        <v>-0.141</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0.2595</v>
+        <v>0.2599</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -15964,13 +17448,13 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>-0.052</v>
+        <v>-0.065</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>0.7113</v>
+        <v>0.6041</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -15996,17 +17480,17 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>K/BB</t>
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>-0.249</v>
+        <v>0.264</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.0322</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H119" s="6" t="inlineStr">
         <is>
@@ -16032,17 +17516,17 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>K/BB</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>0.249</v>
+        <v>-0.218</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>0.0696</v>
+        <v>0.0789</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H120" s="6" t="inlineStr">
         <is>
@@ -16072,13 +17556,13 @@
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>-0.198</v>
+        <v>-0.164</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>0.1502</v>
+        <v>0.1884</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -16104,17 +17588,17 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>-0.191</v>
+        <v>-0.149</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>0.1667</v>
+        <v>0.2311</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -16144,13 +17628,13 @@
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>-0.165</v>
+        <v>-0.117</v>
       </c>
       <c r="F123" s="2" t="n">
-        <v>0.2336</v>
+        <v>0.3497</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -16180,13 +17664,13 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>-0.005</v>
+        <v>0.058</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>0.9736</v>
+        <v>0.6417</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -16432,13 +17916,13 @@
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>-0.326</v>
+        <v>-0.311</v>
       </c>
       <c r="F131" s="2" t="n">
-        <v>0.016</v>
+        <v>0.011</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
@@ -16468,13 +17952,13 @@
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>0.314</v>
+        <v>0.294</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>0.0207</v>
+        <v>0.0165</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
@@ -16504,13 +17988,13 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>-0.302</v>
+        <v>-0.29</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>0.0263</v>
+        <v>0.0182</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
@@ -16540,13 +18024,13 @@
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>0.281</v>
+        <v>0.239</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>0.0398</v>
+        <v>0.0531</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H134" s="6" t="inlineStr">
         <is>
@@ -16612,13 +18096,13 @@
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>-0.133</v>
+        <v>-0.134</v>
       </c>
       <c r="F136" s="2" t="n">
-        <v>0.3365</v>
+        <v>0.2836</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -16648,13 +18132,13 @@
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>-0.106</v>
+        <v>-0.125</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>0.4457</v>
+        <v>0.3189</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -16680,21 +18164,21 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>ERA</t>
+          <t>HR/9</t>
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>-0.21</v>
+        <v>-0.253</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>0.1278</v>
+        <v>0.0403</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="H138" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
+        <v>66</v>
+      </c>
+      <c r="H138" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -16716,17 +18200,17 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>WHIP</t>
+          <t>ERA</t>
         </is>
       </c>
       <c r="E139" s="2" t="n">
-        <v>-0.165</v>
+        <v>-0.2</v>
       </c>
       <c r="F139" s="2" t="n">
-        <v>0.234</v>
+        <v>0.1082</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -16756,13 +18240,13 @@
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>0.157</v>
+        <v>0.185</v>
       </c>
       <c r="F140" s="2" t="n">
-        <v>0.2571</v>
+        <v>0.1377</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -16788,17 +18272,17 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>HR/9</t>
+          <t>WHIP</t>
         </is>
       </c>
       <c r="E141" s="2" t="n">
         <v>-0.154</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>0.2654</v>
+        <v>0.2169</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -16824,17 +18308,17 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>BB/9</t>
+          <t>GB%</t>
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>-0.145</v>
+        <v>0.108</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0.2947</v>
+        <v>0.7128</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -16860,17 +18344,17 @@
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>GB%</t>
+          <t>BB/9</t>
         </is>
       </c>
       <c r="E143" s="2" t="n">
-        <v>0.108</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0.7128</v>
+        <v>0.4822</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
@@ -16900,13 +18384,13 @@
         </is>
       </c>
       <c r="E144" s="2" t="n">
-        <v>-0.028</v>
+        <v>0.04</v>
       </c>
       <c r="F144" s="2" t="n">
-        <v>0.8406</v>
+        <v>0.7487</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -19052,7 +20536,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>80 pitchers</t>
+          <t>94 pitchers</t>
         </is>
       </c>
     </row>
@@ -19069,7 +20553,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>79 pitchers</t>
+          <t>93 pitchers</t>
         </is>
       </c>
     </row>
@@ -19086,7 +20570,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>80 pitchers</t>
+          <t>94 pitchers</t>
         </is>
       </c>
     </row>
@@ -19177,21 +20661,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Total pitchers: 81 (NPB=59, KBO=20, CPBL=2)</t>
+          <t>Total pitchers: 95 (NPB=73, KBO=20, CPBL=2)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Asian-born: 59, American crossover: 20</t>
+          <t>Asian-born: 71, American crossover: 21</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pitchers with both Asian + MLB data: 70</t>
+          <t>Pitchers with both Asian + MLB data: 82</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a references list for the roster, rates, and formulas.
Cite the register, birthplace tables, Stats API, Savant, NPB Data Store, bWAR, Pearson, and the clustering method. wOBA and wRC+ are listed as the published formulas and are not computed on this page.

Co-authored-by: colbymorris08 <colbymorris08@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/asian_pitcher_mlb_analysis.xlsx
+++ b/asian_pitcher_mlb_analysis.xlsx
@@ -17937,12 +17937,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17965,154 +17965,256 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MLB Stats API</t>
+          <t>Baseball-Reference Register</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>statsapi.mlb.com — career + yearly pitching stats (IP, ERA, K, BB, HR, GO/AO)</t>
+          <t>standard_pitching tables for pre-move NPB, KBO, and CPBL seasons</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>72 pitchers</t>
+          <t>Asian seasons</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Baseball-Reference Register</t>
+          <t>Baseball-Reference birthplace tables</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>standard_pitching yearly + summary rows — Asian league stats</t>
+          <t>Japan, South Korea, and Taiwan born pitching lists</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>71 pitchers</t>
+          <t>Asian-born roster check</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>bWAR dataset (pybaseball)</t>
+          <t>MLB Stats API</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>bwar_pitch() — career WAR and ERA+ for MLB seasons</t>
+          <t>stats=career and stats=yearByYear, group=pitching. K/9, BB/9, HR/9, WHIP, K/BB from counting stats</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>72 pitchers</t>
+          <t>MLB seasons</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hand-compiled fallback</t>
+          <t>Baseball Savant</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Research-verified stats for pitchers without API coverage</t>
+          <t>Batted-ball leaderboard, 2015-2026. GB% = ground balls / batted balls, weighted by batted balls</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Fills remaining gaps</t>
+          <t>MLB GB%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>NPB Data Store</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>baseball-data-store.com pitch-type pages, ゴロ率, only when the page title matches the season</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>NPB GB%, 2025-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Baseball-Reference bWAR</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>pybaseball bwar_pitch(); career WAR is the sum, ERA+ is the seasonal mean</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>MLB WAR and ERA+</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Pearson (1895); SciPy pearsonr</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Stability when |r| &gt;= 0.50 and p &lt; 0.10</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>All paired windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Pedregosa et al. (2011), scikit-learn</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Average-linkage clustering on 1 - |r|, distance threshold 0.40; pairs at |r| &gt;= 0.75</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Redundancy, six rate stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Cho (2026)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Cross-League Equivalencies: xFIP- translation factor = 1.096</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>NPB -&gt; MLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Cross-League Equivalencies, xFIP- translation factor 1.096. Not the stability result</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Cited only</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Tango, Lichtman, and Dolphin (2007); FanGraphs wOBA</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>The Book; library.fangraphs.com/offense/woba; Guts! weights. Not computed on this page</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>wOBA formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>FanGraphs wRC and wRC+</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>library.fangraphs.com/offense/wrc. Not computed on this page. Outcomes here are ERA+ and bWAR</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>wRC+ formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>METHODOLOGY</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Stability: Pearson r between Asian-league stat and MLB stat (same metric) across time windows</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Windows: Last 1yr Asia vs First 1yr MLB, 2yr/2yr, 3yr/3yr, Career/Career</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Threshold: |r| &gt;= 0.50 and p &lt; 0.10 to qualify as 'stable'</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>p &lt; 0.10 means &lt; 10% probability the correlation arose by chance (null = no relationship)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Redundancy: Pairwise Pearson r on Asian-league metrics only; pairs at |r| &gt;= 0.75; agglomerative clustering at distance 0.40</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Significance: Pearson r between Asian-league metric (each window) and MLB outcome (ERA+, WAR, seasons); p &lt; 0.10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Total pitchers: 73 (NPB=55, KBO=16, CPBL=2)</t>
+          <t>Stability: Pearson r between Asian-league stat and MLB stat (same metric) across time windows</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Asian-born: 49, American crossover: 21</t>
+          <t>Windows: Last 1yr Asia vs First 1yr MLB, 2yr/2yr, 3yr/3yr, Career/Career</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>Threshold: |r| &gt;= 0.50 and p &lt; 0.10 to qualify as 'stable'</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>p &lt; 0.10 means &lt; 10% probability the correlation arose by chance (null = no relationship)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Redundancy: Pairwise Pearson r on Asian-league metrics only; pairs at |r| &gt;= 0.75; agglomerative clustering at distance 0.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Significance: Pearson r between Asian-league metric (each window) and MLB outcome (ERA+, WAR, seasons); p &lt; 0.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total pitchers: 73 (NPB=55, KBO=16, CPBL=2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Asian-born: 49, American crossover: 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Pitchers with both Asian + MLB data: 66</t>
         </is>

</xml_diff>

<commit_message>
Remove the wOBA and wRC+ citations from the source list.
Those formulas are not used in the roster, the rates, or the correlations.

Co-authored-by: colbymorris08 <colbymorris08@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/asian_pitcher_mlb_analysis.xlsx
+++ b/asian_pitcher_mlb_analysis.xlsx
@@ -17937,7 +17937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18115,106 +18115,72 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Tango, Lichtman, and Dolphin (2007); FanGraphs wOBA</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>The Book; library.fangraphs.com/offense/woba; Guts! weights. Not computed on this page</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>wOBA formula</t>
-        </is>
-      </c>
-    </row>
+    <row r="11"/>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>FanGraphs wRC and wRC+</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>library.fangraphs.com/offense/wrc. Not computed on this page. Outcomes here are ERA+ and bWAR</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>wRC+ formula</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>METHODOLOGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Stability: Pearson r between Asian-league stat and MLB stat (same metric) across time windows</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>METHODOLOGY</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Windows: Last 1yr Asia vs First 1yr MLB, 2yr/2yr, 3yr/3yr, Career/Career</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Stability: Pearson r between Asian-league stat and MLB stat (same metric) across time windows</t>
+          <t>Threshold: |r| &gt;= 0.50 and p &lt; 0.10 to qualify as 'stable'</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Windows: Last 1yr Asia vs First 1yr MLB, 2yr/2yr, 3yr/3yr, Career/Career</t>
+          <t>p &lt; 0.10 means &lt; 10% probability the correlation arose by chance (null = no relationship)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Threshold: |r| &gt;= 0.50 and p &lt; 0.10 to qualify as 'stable'</t>
+          <t>Redundancy: Pairwise Pearson r on Asian-league metrics only; pairs at |r| &gt;= 0.75; agglomerative clustering at distance 0.40</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>p &lt; 0.10 means &lt; 10% probability the correlation arose by chance (null = no relationship)</t>
+          <t>Significance: Pearson r between Asian-league metric (each window) and MLB outcome (ERA+, WAR, seasons); p &lt; 0.10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Redundancy: Pairwise Pearson r on Asian-league metrics only; pairs at |r| &gt;= 0.75; agglomerative clustering at distance 0.40</t>
+          <t>Total pitchers: 73 (NPB=55, KBO=16, CPBL=2)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Significance: Pearson r between Asian-league metric (each window) and MLB outcome (ERA+, WAR, seasons); p &lt; 0.10</t>
+          <t>Asian-born: 49, American crossover: 21</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
-        <is>
-          <t>Total pitchers: 73 (NPB=55, KBO=16, CPBL=2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Asian-born: 49, American crossover: 21</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
         <is>
           <t>Pitchers with both Asian + MLB data: 66</t>
         </is>

</xml_diff>